<commit_message>
Regenerate the outside-in samples against main
Re-promoted all 41 companies against the current image (the merged annual-rate
+ consumer-market classifier, tightened), with no provider calls: existing DB
research re-offered, then re-simulated and re-estimated. Rollups rebuilt from
the per-company output - summary.csv, HIGHLIGHTS.md, the review page and the
workbook. check_samples gate passes; 41/41, 0 failures.

Headline unchanged from the prior set: EUR 508m baseline, 16/41 carry sourced
prices (4.5% value-weighted). The #22 regex tightening does not move the
aggregate - the false positives it fixed were all non-price findings.

Tesco falls to a seed price because the DB has no promotable domain-19 price
quantity for it (research.json still carries the Openreach annual rental, but
it is not ingested as a promotable price) - a research/data absence, not a
consumer over-decline. Noted on PR #22.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -1350,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
@@ -1746,10 +1746,10 @@
         <v>2416</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>12503574.71</v>
+        <v>12513665.95</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>2178899.77</v>
+        <v>2181701.1</v>
       </c>
       <c r="J20" s="6">
         <f>IF(H20=0,"",I20/H20)</f>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="P20" s="6" t="n">
-        <v>0.01000000000000001</v>
+        <v>0.008000000000000007</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>17</v>
@@ -2101,10 +2101,10 @@
         <v>2756</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>12439555.25</v>
+        <v>12682976.67</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>1944683.65</v>
+        <v>2001069.05</v>
       </c>
       <c r="J25" s="6">
         <f>IF(H25=0,"",I25/H25)</f>
@@ -2114,13 +2114,13 @@
         <v>2543904</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M25" s="7" t="n">
         <v>24</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>0.368</v>
+        <v>0.325</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.129</v>
+        <v>0.01600000000000001</v>
       </c>
       <c r="Q25" s="4" t="n">
         <v>17</v>
@@ -2314,10 +2314,10 @@
         <v>16670</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>75796128.16</v>
+        <v>76882377.83</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>13595304.8</v>
+        <v>13896847.7</v>
       </c>
       <c r="J28" s="6">
         <f>IF(H28=0,"",I28/H28)</f>
@@ -2327,7 +2327,7 @@
         <v>13712800.45</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M28" s="7" t="n">
         <v>151</v>
@@ -2341,7 +2341,7 @@
         </is>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.03500000000000003</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="4" t="n">
         <v>17</v>
@@ -3024,7 +3024,7 @@
         <v>3920</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>19293297.97</v>
+        <v>20673102.71</v>
       </c>
       <c r="I38" s="5" t="n">
         <v>3541300.92</v>
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="P38" s="6" t="n">
-        <v>0.526</v>
+        <v>0.03100000000000003</v>
       </c>
       <c r="Q38" s="4" t="n">
         <v>17</v>
@@ -4132,7 +4132,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>32</v>
@@ -4360,16 +4360,16 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>12503574.71</v>
+        <v>12513665.95</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0.01000000000000001</v>
+        <v>0.008000000000000007</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.9752</v>
+        <v>0.9744</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>0</v>
@@ -4378,7 +4378,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.0248</v>
+        <v>0.0256</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12439555.25</v>
+        <v>12682976.67</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>0.00907</v>
+        <v>0.00912</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>0.129</v>
+        <v>0.01600000000000001</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0.9622000000000001</v>
+        <v>0.9629</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>0</v>
@@ -4588,7 +4588,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.0378</v>
+        <v>0.0371</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
@@ -4696,13 +4696,13 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>75796128.16</v>
+        <v>76882377.83</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>0.008869999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.03500000000000003</v>
+        <v>0</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0.9993</v>
@@ -5116,16 +5116,16 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>19293297.97</v>
+        <v>20673102.71</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0.00856</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>0.526</v>
+        <v>0.03100000000000003</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9958</v>
       </c>
       <c r="F38" s="6" t="n">
         <v>0</v>
@@ -5134,7 +5134,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.0045</v>
+        <v>0.0042</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies with the region fallback
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated.

Five companies move. E.ON, Heidelberg Materials, Lufthansa and Rio Tinto
go from PARTIAL to COMPLETE; Iberdrola stays COMPLETE with coverage 85%
to 100%. All five gaps were 5G at 100 Mbps in a country with no 5G rate
of its own. The set baseline moves from EUR 591,604,770 to 592,420,324.

The other 45 are unchanged apart from run ids, timestamps and the new
coverage fields, and their research files apart from promotion ids and
row order.

Capgemini, Danone and Nestle stay PARTIAL: their gaps are 10 Gbps DIA and
2.75 Gbps PON backups, above the top tier on any card. So are 15,039 5G
backups sized at 110 and 275 Mbps against a card that stops at 100.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -2101,10 +2101,10 @@
         <v>218</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>1982748.08</v>
+        <v>2039090.83</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>385333.13</v>
+        <v>400973.87</v>
       </c>
       <c r="J25" s="6">
         <f>IF(H25=0,"",I25/H25)</f>
@@ -2120,7 +2120,7 @@
         <v>3</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>0.271</v>
+        <v>0.339</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -2314,10 +2314,10 @@
         <v>829</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>4753299.1</v>
+        <v>4843301.15</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>841150.53</v>
+        <v>866135.1</v>
       </c>
       <c r="J28" s="6">
         <f>IF(H28=0,"",I28/H28)</f>
@@ -2333,7 +2333,7 @@
         <v>8</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>0.266</v>
+        <v>0.332</v>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
@@ -2341,14 +2341,14 @@
         </is>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.05400000000000005</v>
+        <v>0.05200000000000005</v>
       </c>
       <c r="Q28" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -2527,10 +2527,10 @@
         <v>1273</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>6368593.93</v>
+        <v>6526810.95</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>1115196.53</v>
+        <v>1159117.57</v>
       </c>
       <c r="J31" s="6">
         <f>IF(H31=0,"",I31/H31)</f>
@@ -2540,13 +2540,13 @@
         <v>1398312</v>
       </c>
       <c r="L31" s="7" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M31" s="7" t="n">
         <v>15</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>0.263</v>
+        <v>0.33</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
@@ -2554,14 +2554,14 @@
         </is>
       </c>
       <c r="P31" s="6" t="n">
-        <v>0.01100000000000001</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="Q31" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -2669,10 +2669,10 @@
         <v>2762</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>12763405.23</v>
+        <v>13192517.45</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>2020319.55</v>
+        <v>2139441.1</v>
       </c>
       <c r="J33" s="6">
         <f>IF(H33=0,"",I33/H33)</f>
@@ -2682,13 +2682,13 @@
         <v>2550816</v>
       </c>
       <c r="L33" s="7" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M33" s="7" t="n">
         <v>25</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>0.326</v>
+        <v>0.327</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="Q33" s="4" t="n">
         <v>17</v>
@@ -3237,10 +3237,10 @@
         <v>106</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1565947.9</v>
+        <v>1647827.81</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>340933.02</v>
+        <v>363662.88</v>
       </c>
       <c r="J41" s="6">
         <f>IF(H41=0,"",I41/H41)</f>
@@ -3256,7 +3256,7 @@
         <v>2</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>0.275</v>
+        <v>0.344</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -3264,14 +3264,14 @@
         </is>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.04600000000000004</v>
       </c>
       <c r="Q41" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -5209,16 +5209,16 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1982748.08</v>
+        <v>2039090.83</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>0.00958</v>
+        <v>0.01</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0.7707000000000001</v>
+        <v>0.7771</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>0</v>
@@ -5227,7 +5227,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.2293</v>
+        <v>0.2229</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
@@ -5335,16 +5335,16 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>4753299.1</v>
+        <v>4843301.15</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>0.00962</v>
+        <v>0.01</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.05400000000000005</v>
+        <v>0.05200000000000005</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0.8862</v>
+        <v>0.8697</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>0</v>
@@ -5353,7 +5353,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.1138</v>
+        <v>0.1303</v>
       </c>
       <c r="I28" s="6" t="n">
         <v>0</v>
@@ -5461,16 +5461,16 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>6368593.93</v>
+        <v>6526810.95</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>0.00936</v>
+        <v>0.01</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>0.01100000000000001</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>0.8764999999999999</v>
+        <v>0.8794999999999999</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>0</v>
@@ -5479,7 +5479,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.1235</v>
+        <v>0.1205</v>
       </c>
       <c r="I31" s="6" t="n">
         <v>0</v>
@@ -5545,16 +5545,16 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>12763405.23</v>
+        <v>13192517.45</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>0.00915</v>
+        <v>0.01</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.9607</v>
+        <v>0.9294</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -5563,7 +5563,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.0393</v>
+        <v>0.0706</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
@@ -5881,16 +5881,16 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1565947.9</v>
+        <v>1647827.81</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>0.00942</v>
+        <v>0.01</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.04600000000000004</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>0.9387</v>
+        <v>0.9417</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
@@ -5899,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.0613</v>
+        <v>0.0583</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on the median pass and plan-sized backups
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated.

The set baseline moves from EUR 592,420,324 to 621,474,842.

- The median-pass fix adds EUR 16.6M across 35 companies. Priced backups
  rise from 33,669 to 36,545, matching what the passes counted. EUR 10.5M
  of it is Nestle and Danone, whose plants commit 2,062 Mbps under the
  published fraction - just over the card's 2 Gbps tier, and the next
  Ethernet tier is 10 Gbps.
- Plan-sized backups add EUR 12.4M across 11 companies. Unpriced circuits
  fall from 15,220 to 50, and 15,170 backups are reported as carrying less
  than their primary.

49 companies are COMPLETE. Capgemini stays PARTIAL on 10 Gbps DIA backups,
which are left as asked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -752,17 +752,17 @@
         <v>67</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1155783.04</v>
+        <v>1168338.17</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>290919.64</v>
+        <v>294404.94</v>
       </c>
       <c r="J6" s="6">
         <f>IF(H6=0,"",I6/H6)</f>
         <v/>
       </c>
       <c r="K6" s="5" t="n">
-        <v>66921.39</v>
+        <v>68050.33</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>16</v>
@@ -823,26 +823,26 @@
         <v>2255</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>8470761.83</v>
+        <v>8659494.359999999</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>1198325.04</v>
+        <v>1247634.31</v>
       </c>
       <c r="J7" s="6">
         <f>IF(H7=0,"",I7/H7)</f>
         <v/>
       </c>
       <c r="K7" s="5" t="n">
-        <v>2124216</v>
+        <v>2285352</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>0.325</v>
+        <v>0.318</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
         <v>39</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>1008807.12</v>
+        <v>1013354.26</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>244713.67</v>
@@ -1036,10 +1036,10 @@
         <v>1538</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>17418168.34</v>
+        <v>17547599.86</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>3993381.6</v>
+        <v>4029311.79</v>
       </c>
       <c r="J10" s="6">
         <f>IF(H10=0,"",I10/H10)</f>
@@ -1107,10 +1107,10 @@
         <v>13</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>368823.71</v>
+        <v>373694.9</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>96578.98</v>
+        <v>97931.22</v>
       </c>
       <c r="J11" s="6">
         <f>IF(H11=0,"",I11/H11)</f>
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.06200000000000006</v>
+        <v>0.06799999999999995</v>
       </c>
       <c r="Q11" s="4" t="n">
         <v>17</v>
@@ -1188,7 +1188,7 @@
         <v/>
       </c>
       <c r="K12" s="5" t="n">
-        <v>964944</v>
+        <v>965376</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>11</v>
@@ -1249,17 +1249,17 @@
         <v>232</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>5576208.27</v>
+        <v>5788034.84</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1322400.04</v>
+        <v>1381203.09</v>
       </c>
       <c r="J13" s="6">
         <f>IF(H13=0,"",I13/H13)</f>
         <v/>
       </c>
       <c r="K13" s="5" t="n">
-        <v>269280</v>
+        <v>276624</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>11</v>
@@ -1320,23 +1320,23 @@
         <v>2660</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>31340602.89</v>
+        <v>31866716.63</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>7282948.87</v>
+        <v>7428998.04</v>
       </c>
       <c r="J14" s="6">
         <f>IF(H14=0,"",I14/H14)</f>
         <v/>
       </c>
       <c r="K14" s="5" t="n">
-        <v>2754288</v>
+        <v>3026448</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>12</v>
       </c>
       <c r="M14" s="7" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="N14" s="8" t="n">
         <v>0.343</v>
@@ -1391,23 +1391,23 @@
         <v>2268</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>30232716.66</v>
+        <v>30604118.86</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>7176395.92</v>
+        <v>7279497.17</v>
       </c>
       <c r="J15" s="6">
         <f>IF(H15=0,"",I15/H15)</f>
         <v/>
       </c>
       <c r="K15" s="5" t="n">
-        <v>2342304</v>
+        <v>2576016</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>11</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="N15" s="8" t="n">
         <v>0.343</v>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="P15" s="6" t="n">
-        <v>0.04600000000000004</v>
+        <v>0.04500000000000004</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>17</v>
@@ -1462,17 +1462,17 @@
         <v>98</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>2974519.55</v>
+        <v>3059085.94</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>722178.36</v>
+        <v>745653.99</v>
       </c>
       <c r="J16" s="6">
         <f>IF(H16=0,"",I16/H16)</f>
         <v/>
       </c>
       <c r="K16" s="5" t="n">
-        <v>112176</v>
+        <v>112608</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>16</v>
@@ -1533,10 +1533,10 @@
         <v>2266</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>10513193.2</v>
+        <v>11079390.78</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>1568259.8</v>
+        <v>1657249.58</v>
       </c>
       <c r="J17" s="6">
         <f>IF(H17=0,"",I17/H17)</f>
@@ -1546,13 +1546,13 @@
         <v>2492632.28</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>21</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>0.343</v>
+        <v>0.322</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="P17" s="6" t="n">
-        <v>0.02100000000000002</v>
+        <v>0.01800000000000002</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>17</v>
@@ -1604,17 +1604,17 @@
         <v>106</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>4686313.25</v>
+        <v>4949158.97</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1139971.12</v>
+        <v>1212937.1</v>
       </c>
       <c r="J18" s="6">
         <f>IF(H18=0,"",I18/H18)</f>
         <v/>
       </c>
       <c r="K18" s="5" t="n">
-        <v>119376</v>
+        <v>123264</v>
       </c>
       <c r="L18" s="7" t="n">
         <v>15</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0.04100000000000004</v>
+        <v>0.04200000000000004</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>17</v>
@@ -1675,10 +1675,10 @@
         <v>8982</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>37498493.8</v>
+        <v>39900513.72</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>5750801.7</v>
+        <v>6417602.43</v>
       </c>
       <c r="J19" s="6">
         <f>IF(H19=0,"",I19/H19)</f>
@@ -1688,13 +1688,13 @@
         <v>8479296</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>81</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>0.322</v>
+        <v>0.325</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
@@ -1817,23 +1817,23 @@
         <v>1928</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>20946219.21</v>
+        <v>21165209.15</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>4719498.54</v>
+        <v>4780290.14</v>
       </c>
       <c r="J21" s="6">
         <f>IF(H21=0,"",I21/H21)</f>
         <v/>
       </c>
       <c r="K21" s="5" t="n">
-        <v>1926576</v>
+        <v>2032848</v>
       </c>
       <c r="L21" s="7" t="n">
         <v>13</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N21" s="8" t="n">
         <v>0.342</v>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="P21" s="6" t="n">
-        <v>0.233</v>
+        <v>0.229</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>17</v>
@@ -1959,26 +1959,26 @@
         <v>76</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>2570317.18</v>
+        <v>5658568.77</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>674551.38</v>
+        <v>1531850.03</v>
       </c>
       <c r="J23" s="6">
         <f>IF(H23=0,"",I23/H23)</f>
         <v/>
       </c>
       <c r="K23" s="5" t="n">
-        <v>88272</v>
+        <v>89136</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>0.277</v>
+        <v>0.348</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -2030,17 +2030,17 @@
         <v>5600</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>26009043.62</v>
+        <v>26365288.68</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>4295435.95</v>
+        <v>4394329.58</v>
       </c>
       <c r="J24" s="6">
         <f>IF(H24=0,"",I24/H24)</f>
         <v/>
       </c>
       <c r="K24" s="5" t="n">
-        <v>5166576</v>
+        <v>5169168</v>
       </c>
       <c r="L24" s="7" t="n">
         <v>31</v>
@@ -2101,26 +2101,26 @@
         <v>218</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>2039090.83</v>
+        <v>2150717.42</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>400973.87</v>
+        <v>431961.41</v>
       </c>
       <c r="J25" s="6">
         <f>IF(H25=0,"",I25/H25)</f>
         <v/>
       </c>
       <c r="K25" s="5" t="n">
-        <v>239184</v>
+        <v>240048</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>0.339</v>
+        <v>0.34</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
@@ -2172,23 +2172,23 @@
         <v>2914</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>19078295.1</v>
+        <v>19497183.25</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>3748694.84</v>
+        <v>3864978.19</v>
       </c>
       <c r="J26" s="6">
         <f>IF(H26=0,"",I26/H26)</f>
         <v/>
       </c>
       <c r="K26" s="5" t="n">
-        <v>2607264</v>
+        <v>2779632</v>
       </c>
       <c r="L26" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M26" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="N26" s="8" t="n">
         <v>0.336</v>
@@ -2243,10 +2243,10 @@
         <v>1339</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>6075176.94</v>
+        <v>6439084.19</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>946603.5600000001</v>
+        <v>1047624.21</v>
       </c>
       <c r="J27" s="6">
         <f>IF(H27=0,"",I27/H27)</f>
@@ -2256,13 +2256,13 @@
         <v>1263528</v>
       </c>
       <c r="L27" s="7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M27" s="7" t="n">
         <v>13</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>0.325</v>
+        <v>0.327</v>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
@@ -2314,26 +2314,26 @@
         <v>829</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>4843301.15</v>
+        <v>4998477.86</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>866135.1</v>
+        <v>909212.15</v>
       </c>
       <c r="J28" s="6">
         <f>IF(H28=0,"",I28/H28)</f>
         <v/>
       </c>
       <c r="K28" s="5" t="n">
-        <v>772344</v>
+        <v>773208</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M28" s="7" t="n">
         <v>8</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>0.332</v>
+        <v>0.333</v>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
@@ -2341,7 +2341,7 @@
         </is>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.05200000000000005</v>
+        <v>0.05400000000000005</v>
       </c>
       <c r="Q28" s="4" t="n">
         <v>17</v>
@@ -2385,17 +2385,17 @@
         <v>41</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>2240478.99</v>
+        <v>2244653.58</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>547635.2</v>
+        <v>548794.0600000001</v>
       </c>
       <c r="J29" s="6">
         <f>IF(H29=0,"",I29/H29)</f>
         <v/>
       </c>
       <c r="K29" s="5" t="n">
-        <v>36360</v>
+        <v>37656</v>
       </c>
       <c r="L29" s="7" t="n">
         <v>15</v>
@@ -2456,17 +2456,17 @@
         <v>3385</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>36741069.33</v>
+        <v>36794481</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>8410377.789999999</v>
+        <v>8425204.869999999</v>
       </c>
       <c r="J30" s="6">
         <f>IF(H30=0,"",I30/H30)</f>
         <v/>
       </c>
       <c r="K30" s="5" t="n">
-        <v>3491352</v>
+        <v>3492648</v>
       </c>
       <c r="L30" s="7" t="n">
         <v>12</v>
@@ -2527,17 +2527,17 @@
         <v>1273</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>6526810.95</v>
+        <v>6528520.26</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>1159117.57</v>
+        <v>1159592.08</v>
       </c>
       <c r="J31" s="6">
         <f>IF(H31=0,"",I31/H31)</f>
         <v/>
       </c>
       <c r="K31" s="5" t="n">
-        <v>1398312</v>
+        <v>1399176</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>24</v>
@@ -2598,17 +2598,17 @@
         <v>41</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>678127.5</v>
+        <v>682859.98</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>167225.62</v>
+        <v>168539.36</v>
       </c>
       <c r="J32" s="6">
         <f>IF(H32=0,"",I32/H32)</f>
         <v/>
       </c>
       <c r="K32" s="5" t="n">
-        <v>46296</v>
+        <v>47160</v>
       </c>
       <c r="L32" s="7" t="n">
         <v>17</v>
@@ -2669,17 +2669,17 @@
         <v>2762</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>13192517.45</v>
+        <v>13236997.91</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>2139441.1</v>
+        <v>2151788.87</v>
       </c>
       <c r="J33" s="6">
         <f>IF(H33=0,"",I33/H33)</f>
         <v/>
       </c>
       <c r="K33" s="5" t="n">
-        <v>2550816</v>
+        <v>2551248</v>
       </c>
       <c r="L33" s="7" t="n">
         <v>28</v>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n">
-        <v>0.03000000000000003</v>
+        <v>0.03300000000000003</v>
       </c>
       <c r="Q33" s="4" t="n">
         <v>17</v>
@@ -2740,10 +2740,10 @@
         <v>1695</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>9311406.4</v>
+        <v>9757193.560000001</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>1662443.42</v>
+        <v>1786193.94</v>
       </c>
       <c r="J34" s="6">
         <f>IF(H34=0,"",I34/H34)</f>
@@ -2759,7 +2759,7 @@
         <v>16</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>0.331</v>
+        <v>0.333</v>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
@@ -2811,10 +2811,10 @@
         <v>6061</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>26483053.94</v>
+        <v>28128304</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>4137346.29</v>
+        <v>4594067.71</v>
       </c>
       <c r="J35" s="6">
         <f>IF(H35=0,"",I35/H35)</f>
@@ -2824,13 +2824,13 @@
         <v>5725224</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M35" s="7" t="n">
         <v>55</v>
       </c>
       <c r="N35" s="8" t="n">
-        <v>0.324</v>
+        <v>0.326</v>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
@@ -2882,10 +2882,10 @@
         <v>16671</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>76898026.27</v>
+        <v>81967734.19</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>13900745.06</v>
+        <v>15308095.98</v>
       </c>
       <c r="J36" s="6">
         <f>IF(H36=0,"",I36/H36)</f>
@@ -2895,13 +2895,13 @@
         <v>13714242.99</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M36" s="7" t="n">
         <v>151</v>
       </c>
       <c r="N36" s="8" t="n">
-        <v>0.331</v>
+        <v>0.333</v>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
@@ -2953,17 +2953,17 @@
         <v>1491</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>12841768.74</v>
+        <v>12936989.02</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>2610315.04</v>
+        <v>2636748.2</v>
       </c>
       <c r="J37" s="6">
         <f>IF(H37=0,"",I37/H37)</f>
         <v/>
       </c>
       <c r="K37" s="5" t="n">
-        <v>1736354.54</v>
+        <v>1742909.67</v>
       </c>
       <c r="L37" s="7" t="n">
         <v>18</v>
@@ -2972,7 +2972,7 @@
         <v>15</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>0.337</v>
+        <v>0.338</v>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.857</v>
+        <v>0.858</v>
       </c>
       <c r="Q37" s="4" t="n">
         <v>17</v>
@@ -3024,26 +3024,26 @@
         <v>292</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>10223108.34</v>
+        <v>17871409.34</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>2558834.31</v>
+        <v>4682002.66</v>
       </c>
       <c r="J38" s="6">
         <f>IF(H38=0,"",I38/H38)</f>
         <v/>
       </c>
       <c r="K38" s="5" t="n">
-        <v>363300.97</v>
+        <v>368475.3</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M38" s="7" t="n">
         <v>4</v>
       </c>
       <c r="N38" s="8" t="n">
-        <v>0.277</v>
+        <v>0.348</v>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
@@ -3051,14 +3051,14 @@
         </is>
       </c>
       <c r="P38" s="6" t="n">
-        <v>0.02800000000000002</v>
+        <v>0.01800000000000002</v>
       </c>
       <c r="Q38" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>COMPLETE_FOR_DECLARED_SCOPE</t>
         </is>
       </c>
     </row>
@@ -3095,17 +3095,17 @@
         <v>912</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>5595894.56</v>
+        <v>5670614.04</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>945385.78</v>
+        <v>966127.91</v>
       </c>
       <c r="J39" s="6">
         <f>IF(H39=0,"",I39/H39)</f>
         <v/>
       </c>
       <c r="K39" s="5" t="n">
-        <v>985791.53</v>
+        <v>987808.49</v>
       </c>
       <c r="L39" s="7" t="n">
         <v>20</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.506</v>
+        <v>0.522</v>
       </c>
       <c r="Q39" s="4" t="n">
         <v>17</v>
@@ -3166,17 +3166,17 @@
         <v>125</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>4311337.67</v>
+        <v>4486397.41</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>1010965.53</v>
+        <v>1059562.1</v>
       </c>
       <c r="J40" s="6">
         <f>IF(H40=0,"",I40/H40)</f>
         <v/>
       </c>
       <c r="K40" s="5" t="n">
-        <v>151545.27</v>
+        <v>153426.84</v>
       </c>
       <c r="L40" s="7" t="n">
         <v>16</v>
@@ -3185,7 +3185,7 @@
         <v>2</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>0.346</v>
+        <v>0.347</v>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
@@ -3237,17 +3237,17 @@
         <v>106</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1647827.81</v>
+        <v>1668058.94</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>363662.88</v>
+        <v>369279.05</v>
       </c>
       <c r="J41" s="6">
         <f>IF(H41=0,"",I41/H41)</f>
         <v/>
       </c>
       <c r="K41" s="5" t="n">
-        <v>100225.28</v>
+        <v>102859.49</v>
       </c>
       <c r="L41" s="7" t="n">
         <v>19</v>
@@ -3264,7 +3264,7 @@
         </is>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.04600000000000004</v>
+        <v>0.05900000000000005</v>
       </c>
       <c r="Q41" s="4" t="n">
         <v>16</v>
@@ -3308,26 +3308,26 @@
         <v>1419</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>7556159.11</v>
+        <v>7662037.48</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>1186121.05</v>
+        <v>1215512.89</v>
       </c>
       <c r="J42" s="6">
         <f>IF(H42=0,"",I42/H42)</f>
         <v/>
       </c>
       <c r="K42" s="5" t="n">
-        <v>1476670.32</v>
+        <v>1549785.3</v>
       </c>
       <c r="L42" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M42" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N42" s="8" t="n">
-        <v>0.325</v>
+        <v>0.326</v>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="P42" s="6" t="n">
-        <v>0.297</v>
+        <v>0.284</v>
       </c>
       <c r="Q42" s="4" t="n">
         <v>17</v>
@@ -3379,7 +3379,7 @@
         <v>3419</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>12269507.06</v>
+        <v>12286687.93</v>
       </c>
       <c r="I43" s="5" t="n">
         <v>1949285.51</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="P43" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03700000000000003</v>
       </c>
       <c r="Q43" s="4" t="n">
         <v>17</v>
@@ -3450,17 +3450,17 @@
         <v>502</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>12565745.55</v>
+        <v>13615381.15</v>
       </c>
       <c r="I44" s="5" t="n">
-        <v>3124254.27</v>
+        <v>3415633.12</v>
       </c>
       <c r="J44" s="6">
         <f>IF(H44=0,"",I44/H44)</f>
         <v/>
       </c>
       <c r="K44" s="5" t="n">
-        <v>585936</v>
+        <v>591120</v>
       </c>
       <c r="L44" s="7" t="n">
         <v>9</v>
@@ -3592,10 +3592,10 @@
         <v>3940</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>20836017.21</v>
+        <v>21814060.42</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>3553706.38</v>
+        <v>3635322.5</v>
       </c>
       <c r="J46" s="6">
         <f>IF(H46=0,"",I46/H46)</f>
@@ -3605,13 +3605,13 @@
         <v>4337146.55</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M46" s="7" t="n">
         <v>36</v>
       </c>
       <c r="N46" s="8" t="n">
-        <v>0.38</v>
+        <v>0.327</v>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="P46" s="6" t="n">
-        <v>0.04000000000000004</v>
+        <v>0.03500000000000003</v>
       </c>
       <c r="Q46" s="4" t="n">
         <v>17</v>
@@ -3663,7 +3663,7 @@
         <v>3261</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>10963569.13</v>
+        <v>10964340.57</v>
       </c>
       <c r="I47" s="5" t="n">
         <v>1640998.99</v>
@@ -3734,17 +3734,17 @@
         <v>65</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>2792079.65</v>
+        <v>2835989.78</v>
       </c>
       <c r="I48" s="5" t="n">
-        <v>774257.73</v>
+        <v>786447.1800000001</v>
       </c>
       <c r="J48" s="6">
         <f>IF(H48=0,"",I48/H48)</f>
         <v/>
       </c>
       <c r="K48" s="5" t="n">
-        <v>427.59</v>
+        <v>447.93</v>
       </c>
       <c r="L48" s="7" t="n">
         <v>12</v>
@@ -3805,17 +3805,17 @@
         <v>208</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>4696775.78</v>
+        <v>4789794.63</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1090575.47</v>
+        <v>1116397.5</v>
       </c>
       <c r="J49" s="6">
         <f>IF(H49=0,"",I49/H49)</f>
         <v/>
       </c>
       <c r="K49" s="5" t="n">
-        <v>238608</v>
+        <v>239040</v>
       </c>
       <c r="L49" s="7" t="n">
         <v>12</v>
@@ -3824,7 +3824,7 @@
         <v>3</v>
       </c>
       <c r="N49" s="8" t="n">
-        <v>0.345</v>
+        <v>0.346</v>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="P49" s="6" t="n">
-        <v>0.07099999999999995</v>
+        <v>0.07399999999999995</v>
       </c>
       <c r="Q49" s="4" t="n">
         <v>17</v>
@@ -3876,17 +3876,17 @@
         <v>134</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>1880931.46</v>
+        <v>1923460.09</v>
       </c>
       <c r="I50" s="5" t="n">
-        <v>415866.18</v>
+        <v>427672.13</v>
       </c>
       <c r="J50" s="6">
         <f>IF(H50=0,"",I50/H50)</f>
         <v/>
       </c>
       <c r="K50" s="5" t="n">
-        <v>112016.49</v>
+        <v>118790.16</v>
       </c>
       <c r="L50" s="7" t="n">
         <v>17</v>
@@ -3947,23 +3947,23 @@
         <v>1089</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>21822847.1</v>
+        <v>22704990.14</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>5525188.64</v>
+        <v>5770071.55</v>
       </c>
       <c r="J51" s="6">
         <f>IF(H51=0,"",I51/H51)</f>
         <v/>
       </c>
       <c r="K51" s="5" t="n">
-        <v>927805.13</v>
+        <v>1077578.58</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M51" s="7" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="N51" s="8" t="n">
         <v>0.346</v>
@@ -4018,10 +4018,10 @@
         <v>835</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>4440110.64</v>
+        <v>4699559.06</v>
       </c>
       <c r="I52" s="5" t="n">
-        <v>813190.78</v>
+        <v>885213.67</v>
       </c>
       <c r="J52" s="6">
         <f>IF(H52=0,"",I52/H52)</f>
@@ -4031,13 +4031,13 @@
         <v>686712.52</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M52" s="7" t="n">
         <v>8</v>
       </c>
       <c r="N52" s="8" t="n">
-        <v>0.334</v>
+        <v>0.335</v>
       </c>
       <c r="O52" s="4" t="inlineStr">
         <is>
@@ -4089,17 +4089,17 @@
         <v>181</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>5924550.33</v>
+        <v>6284919.48</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>1445249.82</v>
+        <v>1545288.3</v>
       </c>
       <c r="J53" s="6">
         <f>IF(H53=0,"",I53/H53)</f>
         <v/>
       </c>
       <c r="K53" s="5" t="n">
-        <v>208152</v>
+        <v>213336</v>
       </c>
       <c r="L53" s="7" t="n">
         <v>12</v>
@@ -4160,10 +4160,10 @@
         <v>1363</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>5935359.84</v>
+        <v>6395969.65</v>
       </c>
       <c r="I54" s="5" t="n">
-        <v>1204942.01</v>
+        <v>1332807.29</v>
       </c>
       <c r="J54" s="6">
         <f>IF(H54=0,"",I54/H54)</f>
@@ -4173,13 +4173,13 @@
         <v>758181.9</v>
       </c>
       <c r="L54" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M54" s="7" t="n">
         <v>13</v>
       </c>
       <c r="N54" s="8" t="n">
-        <v>0.337</v>
+        <v>0.338</v>
       </c>
       <c r="O54" s="4" t="inlineStr">
         <is>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1155783.04</v>
+        <v>1168338.17</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>0.01</v>
@@ -4420,7 +4420,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.8686</v>
+        <v>0.866</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -4429,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.1314</v>
+        <v>0.134</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>0</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8470761.83</v>
+        <v>8659494.359999999</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>0.01</v>
@@ -4462,7 +4462,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.9452</v>
+        <v>0.9251</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -4471,7 +4471,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.0548</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>0</v>
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1008807.12</v>
+        <v>1013354.26</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0.01</v>
@@ -4546,7 +4546,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.9538</v>
+        <v>0.954</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -4555,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.0462</v>
+        <v>0.046</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0</v>
@@ -4579,7 +4579,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>17418168.34</v>
+        <v>17547599.86</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>0.009979999999999999</v>
@@ -4588,7 +4588,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.9345</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -4597,7 +4597,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.0655</v>
+        <v>0.065</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
@@ -4621,16 +4621,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>368823.71</v>
+        <v>373694.9</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.06200000000000006</v>
+        <v>0.06799999999999995</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.8407</v>
+        <v>0.8428</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>0</v>
@@ -4639,7 +4639,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.1593</v>
+        <v>0.1572</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>0</v>
@@ -4666,7 +4666,7 @@
         <v>13972078.09</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>0.00987</v>
+        <v>0.009860000000000001</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5576208.27</v>
+        <v>5788034.84</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>0.01</v>
@@ -4714,7 +4714,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8025</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -4723,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.192</v>
+        <v>0.1975</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>0</v>
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>31340602.89</v>
+        <v>31866716.63</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>0.01</v>
@@ -4756,7 +4756,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0.9401</v>
+        <v>0.9265</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>0</v>
@@ -4765,7 +4765,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.0599</v>
+        <v>0.0735</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>0</v>
@@ -4789,16 +4789,16 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>30232716.66</v>
+        <v>30604118.86</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.04600000000000004</v>
+        <v>0.04500000000000004</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9595</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>0</v>
@@ -4807,7 +4807,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.0287</v>
+        <v>0.0405</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0</v>
@@ -4831,7 +4831,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>2974519.55</v>
+        <v>3059085.94</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>0.01</v>
@@ -4840,7 +4840,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0.8901</v>
+        <v>0.8885</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>0</v>
@@ -4849,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.1099</v>
+        <v>0.1115</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>0</v>
@@ -4873,16 +4873,16 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>10513193.2</v>
+        <v>11079390.78</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.008279999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.02100000000000002</v>
+        <v>0.01800000000000002</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>0.9981</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -4891,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.0019</v>
+        <v>0.0529</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0</v>
@@ -4915,16 +4915,16 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>4686313.25</v>
+        <v>4949158.97</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.00906</v>
+        <v>0.00903</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.04100000000000004</v>
+        <v>0.04200000000000004</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>0.8436</v>
+        <v>0.833</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>0</v>
@@ -4933,7 +4933,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.1564</v>
+        <v>0.167</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
@@ -4957,16 +4957,16 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>37498493.8</v>
+        <v>39900513.72</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.008359999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="D19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.9971</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
@@ -4975,7 +4975,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.0029</v>
+        <v>0.063</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
@@ -5041,16 +5041,16 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>20946219.21</v>
+        <v>21165209.15</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>0.233</v>
+        <v>0.229</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.96</v>
+        <v>0.9500999999999999</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
@@ -5059,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.04</v>
+        <v>0.0499</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
@@ -5125,16 +5125,16 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2570317.18</v>
+        <v>5658568.77</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>0.009689999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="D23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.9733000000000001</v>
+        <v>0.9747</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
@@ -5143,7 +5143,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.0267</v>
+        <v>0.0253</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>26009043.62</v>
+        <v>26365288.68</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>0.01</v>
@@ -5176,7 +5176,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>0.913</v>
+        <v>0.9105</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>0</v>
@@ -5185,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.0895</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>0</v>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2039090.83</v>
+        <v>2150717.42</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>0.01</v>
@@ -5218,7 +5218,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0.7771</v>
+        <v>0.7745</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>0</v>
@@ -5227,7 +5227,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.2229</v>
+        <v>0.2255</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>19078295.1</v>
+        <v>19497183.25</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>0.01</v>
@@ -5260,7 +5260,7 @@
         <v>0.004000000000000004</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>0.9681</v>
+        <v>0.9486</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>0</v>
@@ -5269,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.0319</v>
+        <v>0.0514</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0</v>
@@ -5293,16 +5293,16 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6075176.94</v>
+        <v>6439084.19</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>0.008579999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="D27" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1</v>
+        <v>0.9435</v>
       </c>
       <c r="F27" s="6" t="n">
         <v>0</v>
@@ -5311,7 +5311,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0</v>
+        <v>0.0565</v>
       </c>
       <c r="I27" s="6" t="n">
         <v>0</v>
@@ -5335,16 +5335,16 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>4843301.15</v>
+        <v>4998477.86</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.05200000000000005</v>
+        <v>0.05400000000000005</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0.8697</v>
+        <v>0.8671</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>0</v>
@@ -5353,7 +5353,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.1303</v>
+        <v>0.1329</v>
       </c>
       <c r="I28" s="6" t="n">
         <v>0</v>
@@ -5377,7 +5377,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2240478.99</v>
+        <v>2244653.58</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>0.01</v>
@@ -5386,7 +5386,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>0.9539</v>
+        <v>0.9520999999999999</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>0</v>
@@ -5395,7 +5395,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0.0461</v>
+        <v>0.0479</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>36741069.33</v>
+        <v>36794481</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>0.01</v>
@@ -5428,7 +5428,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0.9526</v>
+        <v>0.9520999999999999</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>0</v>
@@ -5437,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.0474</v>
+        <v>0.0479</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>0</v>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>6526810.95</v>
+        <v>6528520.26</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>0.01</v>
@@ -5470,7 +5470,7 @@
         <v>0.01000000000000001</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.8793</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>0</v>
@@ -5479,7 +5479,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.1205</v>
+        <v>0.1207</v>
       </c>
       <c r="I31" s="6" t="n">
         <v>0</v>
@@ -5503,7 +5503,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>678127.5</v>
+        <v>682859.98</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>0.01</v>
@@ -5512,7 +5512,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.8857</v>
+        <v>0.882</v>
       </c>
       <c r="F32" s="6" t="n">
         <v>0</v>
@@ -5521,7 +5521,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.1143</v>
+        <v>0.118</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0</v>
@@ -5545,16 +5545,16 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>13192517.45</v>
+        <v>13236997.91</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>0.03000000000000003</v>
+        <v>0.03300000000000003</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.9294</v>
+        <v>0.9286</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -5563,7 +5563,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.0706</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
@@ -5587,16 +5587,16 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9311406.4</v>
+        <v>9757193.560000001</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>0.00907</v>
+        <v>0.01</v>
       </c>
       <c r="D34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>0.996</v>
+        <v>0.9505</v>
       </c>
       <c r="F34" s="6" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0495</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>0</v>
@@ -5629,16 +5629,16 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>26483053.94</v>
+        <v>28128304</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0.00852</v>
+        <v>0.01</v>
       </c>
       <c r="D35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>0.9943</v>
+        <v>0.9362</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -5647,7 +5647,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0.0057</v>
+        <v>0.0638</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>0</v>
@@ -5671,16 +5671,16 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>76898026.27</v>
+        <v>81967734.19</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0.0089</v>
+        <v>0.01</v>
       </c>
       <c r="D36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0.9992</v>
+        <v>0.9374</v>
       </c>
       <c r="F36" s="6" t="n">
         <v>0</v>
@@ -5689,7 +5689,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.0008</v>
+        <v>0.0626</v>
       </c>
       <c r="I36" s="6" t="n">
         <v>0</v>
@@ -5713,16 +5713,16 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>12841768.74</v>
+        <v>12936989.02</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>0.857</v>
+        <v>0.858</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0.9405</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
@@ -5731,7 +5731,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0.0595</v>
+        <v>0.061</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0</v>
@@ -5755,16 +5755,16 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>10223108.34</v>
+        <v>17871409.34</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0.00984</v>
+        <v>0.01</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>0.02800000000000002</v>
+        <v>0.01800000000000002</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.9073</v>
+        <v>0.9358</v>
       </c>
       <c r="F38" s="6" t="n">
         <v>0</v>
@@ -5773,7 +5773,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.0927</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>
@@ -5797,16 +5797,16 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5595894.56</v>
+        <v>5670614.04</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>0.506</v>
+        <v>0.522</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9324</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>0</v>
@@ -5815,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.063</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>4311337.67</v>
+        <v>4486397.41</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>0.01</v>
@@ -5848,7 +5848,7 @@
         <v>0</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0.8178</v>
+        <v>0.8118</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
@@ -5857,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0.1822</v>
+        <v>0.1882</v>
       </c>
       <c r="I40" s="6" t="n">
         <v>0</v>
@@ -5881,16 +5881,16 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1647827.81</v>
+        <v>1668058.94</v>
       </c>
       <c r="C41" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>0.04600000000000004</v>
+        <v>0.05900000000000005</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>0.9417</v>
+        <v>0.9345</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
@@ -5899,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.0583</v>
+        <v>0.0655</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>
@@ -5923,16 +5923,16 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7556159.11</v>
+        <v>7662037.48</v>
       </c>
       <c r="C42" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>0.297</v>
+        <v>0.284</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0.9688</v>
+        <v>0.9554</v>
       </c>
       <c r="F42" s="6" t="n">
         <v>0</v>
@@ -5941,7 +5941,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.0312</v>
+        <v>0.0446</v>
       </c>
       <c r="I42" s="6" t="n">
         <v>0</v>
@@ -5965,13 +5965,13 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>12269507.06</v>
+        <v>12286687.93</v>
       </c>
       <c r="C43" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03700000000000003</v>
       </c>
       <c r="E43" s="6" t="n">
         <v>0.9638</v>
@@ -6007,7 +6007,7 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>12565745.55</v>
+        <v>13615381.15</v>
       </c>
       <c r="C44" s="6" t="n">
         <v>0.01</v>
@@ -6016,7 +6016,7 @@
         <v>0.03800000000000003</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>0.6236</v>
+        <v>0.6418</v>
       </c>
       <c r="F44" s="6" t="n">
         <v>0</v>
@@ -6025,7 +6025,7 @@
         <v>0</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0.3764</v>
+        <v>0.3582</v>
       </c>
       <c r="I44" s="6" t="n">
         <v>0</v>
@@ -6091,16 +6091,16 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>20836017.21</v>
+        <v>21814060.42</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>0.00881</v>
+        <v>0.01</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>0.04000000000000004</v>
+        <v>0.03500000000000003</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>0.9954</v>
+        <v>0.9508</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>0</v>
@@ -6109,7 +6109,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.0046</v>
+        <v>0.0492</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>0</v>
@@ -6133,7 +6133,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>10963569.13</v>
+        <v>10964340.57</v>
       </c>
       <c r="C47" s="6" t="n">
         <v>0.01</v>
@@ -6175,7 +6175,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>2792079.65</v>
+        <v>2835989.78</v>
       </c>
       <c r="C48" s="6" t="n">
         <v>0.01</v>
@@ -6184,7 +6184,7 @@
         <v>0.007000000000000006</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>0.9253</v>
+        <v>0.9179</v>
       </c>
       <c r="F48" s="6" t="n">
         <v>0</v>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.0747</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
@@ -6217,16 +6217,16 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>4696775.78</v>
+        <v>4789794.63</v>
       </c>
       <c r="C49" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>0.07099999999999995</v>
+        <v>0.07399999999999995</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>0.8174</v>
+        <v>0.8207</v>
       </c>
       <c r="F49" s="6" t="n">
         <v>0</v>
@@ -6235,7 +6235,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.1826</v>
+        <v>0.1793</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>0</v>
@@ -6259,7 +6259,7 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>1880931.46</v>
+        <v>1923460.09</v>
       </c>
       <c r="C50" s="6" t="n">
         <v>0.01</v>
@@ -6268,7 +6268,7 @@
         <v>0</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>0.9462</v>
+        <v>0.9253</v>
       </c>
       <c r="F50" s="6" t="n">
         <v>0</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.0538</v>
+        <v>0.0747</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>0</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>21822847.1</v>
+        <v>22704990.14</v>
       </c>
       <c r="C51" s="6" t="n">
         <v>0.01</v>
@@ -6310,7 +6310,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>0.9510999999999999</v>
+        <v>0.9141</v>
       </c>
       <c r="F51" s="6" t="n">
         <v>0</v>
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.0489</v>
+        <v>0.0859</v>
       </c>
       <c r="I51" s="6" t="n">
         <v>0</v>
@@ -6343,16 +6343,16 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>4440110.64</v>
+        <v>4699559.06</v>
       </c>
       <c r="C52" s="6" t="n">
-        <v>0.009090000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="D52" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>0.9961</v>
+        <v>0.9411</v>
       </c>
       <c r="F52" s="6" t="n">
         <v>0</v>
@@ -6361,7 +6361,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.0039</v>
+        <v>0.0589</v>
       </c>
       <c r="I52" s="6" t="n">
         <v>0</v>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>5924550.33</v>
+        <v>6284919.48</v>
       </c>
       <c r="C53" s="6" t="n">
         <v>0.01</v>
@@ -6394,7 +6394,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>0.7744</v>
+        <v>0.7688</v>
       </c>
       <c r="F53" s="6" t="n">
         <v>0</v>
@@ -6403,7 +6403,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.2256</v>
+        <v>0.2312</v>
       </c>
       <c r="I53" s="6" t="n">
         <v>0</v>
@@ -6427,16 +6427,16 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>5935359.84</v>
+        <v>6395969.65</v>
       </c>
       <c r="C54" s="6" t="n">
-        <v>0.0091</v>
+        <v>0.01</v>
       </c>
       <c r="D54" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>0.9818</v>
+        <v>0.9111</v>
       </c>
       <c r="F54" s="6" t="n">
         <v>0</v>
@@ -6445,7 +6445,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.0182</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="I54" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on the filled Ethernet card
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated.

The set baseline moves from EUR 621,474,842 to 610,696,962. 24 companies
fall and none rise; Nestle (-6.2M) and Danone (-2.5M) are most of it. Of
the 431 circuits that needed 2 to 10 Gbps, 382 move to the next 1 Gbps
step, 32 now match a tier exactly, and the 17 needing 9,500 Mbps or more
stay at 10 Gbps. 49 companies are COMPLETE, as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -681,10 +681,10 @@
         <v>156</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>3051904.55</v>
+        <v>2905267.73</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>829346.13</v>
+        <v>788639.74</v>
       </c>
       <c r="J5" s="6">
         <f>IF(H5=0,"",I5/H5)</f>
@@ -894,10 +894,10 @@
         <v>78</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>5188847.93</v>
+        <v>4831236.05</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>1347130.83</v>
+        <v>1247857.77</v>
       </c>
       <c r="J8" s="6">
         <f>IF(H8=0,"",I8/H8)</f>
@@ -965,7 +965,7 @@
         <v>39</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>1013354.26</v>
+        <v>992580.71</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>244713.67</v>
@@ -1036,10 +1036,10 @@
         <v>1538</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>17547599.86</v>
+        <v>17529277.02</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>4029311.79</v>
+        <v>4024225.37</v>
       </c>
       <c r="J10" s="6">
         <f>IF(H10=0,"",I10/H10)</f>
@@ -1178,10 +1178,10 @@
         <v>932</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>13972078.09</v>
+        <v>13832111.34</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>3400769.98</v>
+        <v>3361915.21</v>
       </c>
       <c r="J12" s="6">
         <f>IF(H12=0,"",I12/H12)</f>
@@ -1391,10 +1391,10 @@
         <v>2268</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>30604118.86</v>
+        <v>30585796.02</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>7279497.17</v>
+        <v>7274410.75</v>
       </c>
       <c r="J15" s="6">
         <f>IF(H15=0,"",I15/H15)</f>
@@ -1604,10 +1604,10 @@
         <v>106</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>4949158.97</v>
+        <v>4759969.53</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1212937.1</v>
+        <v>1160418.11</v>
       </c>
       <c r="J18" s="6">
         <f>IF(H18=0,"",I18/H18)</f>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0.04200000000000004</v>
+        <v>0.03700000000000003</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>17</v>
@@ -1817,10 +1817,10 @@
         <v>1928</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>21165209.15</v>
+        <v>21150658.08</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>4780290.14</v>
+        <v>4776250.77</v>
       </c>
       <c r="J21" s="6">
         <f>IF(H21=0,"",I21/H21)</f>
@@ -1888,10 +1888,10 @@
         <v>1769</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>11746529.67</v>
+        <v>11633057.47</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>2607276.05</v>
+        <v>2575776.17</v>
       </c>
       <c r="J22" s="6">
         <f>IF(H22=0,"",I22/H22)</f>
@@ -1959,10 +1959,10 @@
         <v>76</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>5658568.77</v>
+        <v>3147880.1</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>1531850.03</v>
+        <v>834882.85</v>
       </c>
       <c r="J23" s="6">
         <f>IF(H23=0,"",I23/H23)</f>
@@ -1972,13 +1972,13 @@
         <v>89136</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>0.348</v>
+        <v>0.347</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
@@ -2030,10 +2030,10 @@
         <v>5600</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>26365288.68</v>
+        <v>26337114.27</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>4394329.58</v>
+        <v>4386508.36</v>
       </c>
       <c r="J24" s="6">
         <f>IF(H24=0,"",I24/H24)</f>
@@ -2314,10 +2314,10 @@
         <v>829</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>4998477.86</v>
+        <v>4934058.18</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>909212.15</v>
+        <v>891329.25</v>
       </c>
       <c r="J28" s="6">
         <f>IF(H28=0,"",I28/H28)</f>
@@ -2341,7 +2341,7 @@
         </is>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.05400000000000005</v>
+        <v>0.05500000000000005</v>
       </c>
       <c r="Q28" s="4" t="n">
         <v>17</v>
@@ -2385,10 +2385,10 @@
         <v>41</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>2244653.58</v>
+        <v>2157714.62</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>548794.0600000001</v>
+        <v>524659.8100000001</v>
       </c>
       <c r="J29" s="6">
         <f>IF(H29=0,"",I29/H29)</f>
@@ -2669,10 +2669,10 @@
         <v>2762</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>13236997.91</v>
+        <v>13002327.96</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>2151788.87</v>
+        <v>2086644.49</v>
       </c>
       <c r="J33" s="6">
         <f>IF(H33=0,"",I33/H33)</f>
@@ -2688,7 +2688,7 @@
         <v>25</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>0.327</v>
+        <v>0.326</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03400000000000003</v>
       </c>
       <c r="Q33" s="4" t="n">
         <v>17</v>
@@ -2740,10 +2740,10 @@
         <v>1695</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>9757193.560000001</v>
+        <v>9457122.9</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>1786193.94</v>
+        <v>1702894.32</v>
       </c>
       <c r="J34" s="6">
         <f>IF(H34=0,"",I34/H34)</f>
@@ -2759,7 +2759,7 @@
         <v>16</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>0.333</v>
+        <v>0.332</v>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
@@ -3024,10 +3024,10 @@
         <v>292</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>17871409.34</v>
+        <v>11678474.51</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>4682002.66</v>
+        <v>2962843.96</v>
       </c>
       <c r="J38" s="6">
         <f>IF(H38=0,"",I38/H38)</f>
@@ -3037,13 +3037,13 @@
         <v>368475.3</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M38" s="7" t="n">
         <v>4</v>
       </c>
       <c r="N38" s="8" t="n">
-        <v>0.348</v>
+        <v>0.347</v>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="P38" s="6" t="n">
-        <v>0.01800000000000002</v>
+        <v>0.02600000000000002</v>
       </c>
       <c r="Q38" s="4" t="n">
         <v>17</v>
@@ -3095,10 +3095,10 @@
         <v>912</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>5670614.04</v>
+        <v>5634188.81</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>966127.91</v>
+        <v>956016.26</v>
       </c>
       <c r="J39" s="6">
         <f>IF(H39=0,"",I39/H39)</f>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.522</v>
+        <v>0.261</v>
       </c>
       <c r="Q39" s="4" t="n">
         <v>17</v>
@@ -3166,10 +3166,10 @@
         <v>125</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>4486397.41</v>
+        <v>4424642.29</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>1059562.1</v>
+        <v>1042418.88</v>
       </c>
       <c r="J40" s="6">
         <f>IF(H40=0,"",I40/H40)</f>
@@ -3185,7 +3185,7 @@
         <v>2</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>0.347</v>
+        <v>0.346</v>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
@@ -3237,10 +3237,10 @@
         <v>106</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1668058.94</v>
+        <v>1634821.48</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>369279.05</v>
+        <v>360052.33</v>
       </c>
       <c r="J41" s="6">
         <f>IF(H41=0,"",I41/H41)</f>
@@ -3264,7 +3264,7 @@
         </is>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.05900000000000005</v>
+        <v>0.06100000000000005</v>
       </c>
       <c r="Q41" s="4" t="n">
         <v>16</v>
@@ -3379,7 +3379,7 @@
         <v>3419</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>12286687.93</v>
+        <v>12272260.2</v>
       </c>
       <c r="I43" s="5" t="n">
         <v>1949285.51</v>
@@ -3663,7 +3663,7 @@
         <v>3261</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>10964340.57</v>
+        <v>10954055.03</v>
       </c>
       <c r="I47" s="5" t="n">
         <v>1640998.99</v>
@@ -3734,10 +3734,10 @@
         <v>65</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>2835989.78</v>
+        <v>2779745.33</v>
       </c>
       <c r="I48" s="5" t="n">
-        <v>786447.1800000001</v>
+        <v>770833.72</v>
       </c>
       <c r="J48" s="6">
         <f>IF(H48=0,"",I48/H48)</f>
@@ -4089,10 +4089,10 @@
         <v>181</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>6284919.48</v>
+        <v>6228675.04</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>1545288.3</v>
+        <v>1529674.84</v>
       </c>
       <c r="J53" s="6">
         <f>IF(H53=0,"",I53/H53)</f>
@@ -4160,10 +4160,10 @@
         <v>1363</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>6395969.65</v>
+        <v>6323454.09</v>
       </c>
       <c r="I54" s="5" t="n">
-        <v>1332807.29</v>
+        <v>1312676.97</v>
       </c>
       <c r="J54" s="6">
         <f>IF(H54=0,"",I54/H54)</f>
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3051904.55</v>
+        <v>2905267.73</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>0.01</v>
@@ -4378,7 +4378,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.9592000000000001</v>
+        <v>0.9571</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -4387,7 +4387,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.0408</v>
+        <v>0.0429</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>0</v>
@@ -4495,10 +4495,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5188847.93</v>
+        <v>4831236.05</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.009889999999999999</v>
+        <v>0.00988</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0.005000000000000004</v>
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1013354.26</v>
+        <v>992580.71</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0.01</v>
@@ -4546,7 +4546,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.954</v>
+        <v>0.953</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -4555,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.046</v>
+        <v>0.047</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0</v>
@@ -4579,7 +4579,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>17547599.86</v>
+        <v>17529277.02</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>0.009979999999999999</v>
@@ -4588,7 +4588,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9349</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -4597,7 +4597,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.065</v>
+        <v>0.06510000000000001</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
@@ -4663,7 +4663,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>13972078.09</v>
+        <v>13832111.34</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0.009860000000000001</v>
@@ -4672,7 +4672,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.9744</v>
+        <v>0.9741</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>0</v>
@@ -4681,7 +4681,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.0256</v>
+        <v>0.0259</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0</v>
@@ -4789,7 +4789,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>30604118.86</v>
+        <v>30585796.02</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>0.01</v>
@@ -4915,16 +4915,16 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>4949158.97</v>
+        <v>4759969.53</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.00903</v>
+        <v>0.00899</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.04200000000000004</v>
+        <v>0.03700000000000003</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>0.833</v>
+        <v>0.8263</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>0</v>
@@ -4933,7 +4933,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.167</v>
+        <v>0.1737</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
@@ -5041,7 +5041,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>21165209.15</v>
+        <v>21150658.08</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>0.01</v>
@@ -5050,7 +5050,7 @@
         <v>0.229</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.9500999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
@@ -5059,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.0499</v>
+        <v>0.05</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11746529.67</v>
+        <v>11633057.47</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>0.01</v>
@@ -5092,7 +5092,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.9429</v>
+        <v>0.9423</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>0</v>
@@ -5101,7 +5101,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.0571</v>
+        <v>0.0577</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>5658568.77</v>
+        <v>3147880.1</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>0.01</v>
@@ -5134,7 +5134,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.9747</v>
+        <v>0.9545</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
@@ -5143,7 +5143,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.0253</v>
+        <v>0.0455</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>26365288.68</v>
+        <v>26337114.27</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>0.01</v>
@@ -5176,7 +5176,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>0.9105</v>
+        <v>0.9104</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>0</v>
@@ -5185,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.0895</v>
+        <v>0.0896</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>0</v>
@@ -5335,16 +5335,16 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>4998477.86</v>
+        <v>4934058.18</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.05400000000000005</v>
+        <v>0.05500000000000005</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0.8671</v>
+        <v>0.8653999999999999</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>0</v>
@@ -5353,7 +5353,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.1329</v>
+        <v>0.1346</v>
       </c>
       <c r="I28" s="6" t="n">
         <v>0</v>
@@ -5377,7 +5377,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2244653.58</v>
+        <v>2157714.62</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>0.01</v>
@@ -5386,7 +5386,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>0.9520999999999999</v>
+        <v>0.9502</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>0</v>
@@ -5395,7 +5395,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0.0479</v>
+        <v>0.0498</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
@@ -5545,16 +5545,16 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>13236997.91</v>
+        <v>13002327.96</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>0.03300000000000003</v>
+        <v>0.03400000000000003</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.9286</v>
+        <v>0.9273</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -5563,7 +5563,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.0727</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9757193.560000001</v>
+        <v>9457122.9</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>0.01</v>
@@ -5596,7 +5596,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>0.9505</v>
+        <v>0.9489</v>
       </c>
       <c r="F34" s="6" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.0495</v>
+        <v>0.0511</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>0</v>
@@ -5755,16 +5755,16 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>17871409.34</v>
+        <v>11678474.51</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>0.01800000000000002</v>
+        <v>0.02600000000000002</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.9358</v>
+        <v>0.9016999999999999</v>
       </c>
       <c r="F38" s="6" t="n">
         <v>0</v>
@@ -5773,7 +5773,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0983</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>
@@ -5797,16 +5797,16 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5670614.04</v>
+        <v>5634188.81</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>0.522</v>
+        <v>0.261</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0.9324</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>0</v>
@@ -5815,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.068</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>4486397.41</v>
+        <v>4424642.29</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>0.01</v>
@@ -5848,7 +5848,7 @@
         <v>0</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0.8118</v>
+        <v>0.8092</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
@@ -5857,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0.1882</v>
+        <v>0.1908</v>
       </c>
       <c r="I40" s="6" t="n">
         <v>0</v>
@@ -5881,16 +5881,16 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1668058.94</v>
+        <v>1634821.48</v>
       </c>
       <c r="C41" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>0.05900000000000005</v>
+        <v>0.06100000000000005</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>0.9345</v>
+        <v>0.9332</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
@@ -5899,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.0655</v>
+        <v>0.0668</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>
@@ -5965,7 +5965,7 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>12286687.93</v>
+        <v>12272260.2</v>
       </c>
       <c r="C43" s="6" t="n">
         <v>0.01</v>
@@ -6133,7 +6133,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>10964340.57</v>
+        <v>10954055.03</v>
       </c>
       <c r="C47" s="6" t="n">
         <v>0.01</v>
@@ -6175,7 +6175,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>2835989.78</v>
+        <v>2779745.33</v>
       </c>
       <c r="C48" s="6" t="n">
         <v>0.01</v>
@@ -6184,7 +6184,7 @@
         <v>0.007000000000000006</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>0.9179</v>
+        <v>0.9162</v>
       </c>
       <c r="F48" s="6" t="n">
         <v>0</v>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.0838</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>6284919.48</v>
+        <v>6228675.04</v>
       </c>
       <c r="C53" s="6" t="n">
         <v>0.01</v>
@@ -6394,7 +6394,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>0.7688</v>
+        <v>0.7667</v>
       </c>
       <c r="F53" s="6" t="n">
         <v>0</v>
@@ -6403,7 +6403,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.2312</v>
+        <v>0.2333</v>
       </c>
       <c r="I53" s="6" t="n">
         <v>0</v>
@@ -6427,7 +6427,7 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>6395969.65</v>
+        <v>6323454.09</v>
       </c>
       <c r="C54" s="6" t="n">
         <v>0.01</v>
@@ -6436,7 +6436,7 @@
         <v>0</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>0.9111</v>
+        <v>0.9101</v>
       </c>
       <c r="F54" s="6" t="n">
         <v>0</v>
@@ -6445,7 +6445,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="I54" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on the approved researched prices
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The decisions held through the
run - 28 approved, 19 revoked, 12 undecided after it as before - and
research challenged five of them with other figures, which the card did
not take.

The set baseline moves from EUR 610,696,962 to 584,087,950 (-26.6M,
-4.4%) across 40 companies, exactly what the review predicted. McDonald's
-16.1M, Tesco -2.7M, Boots -1.5M; Fresenius +0.6M where the US DIA 100
median sits above the seed it replaced. Researched prices now carry 22.5%
of priced value, up from 4.0%, in 43 companies. 49 stay COMPLETE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -681,10 +681,10 @@
         <v>156</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>2905267.73</v>
+        <v>2907843.4</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>788639.74</v>
+        <v>789354.75</v>
       </c>
       <c r="J5" s="6">
         <f>IF(H5=0,"",I5/H5)</f>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0</v>
+        <v>0.09799999999999998</v>
       </c>
       <c r="Q5" s="4" t="n">
         <v>17</v>
@@ -752,10 +752,10 @@
         <v>67</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1168338.17</v>
+        <v>1159918.54</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>294404.94</v>
+        <v>292067.65</v>
       </c>
       <c r="J6" s="6">
         <f>IF(H6=0,"",I6/H6)</f>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0</v>
+        <v>0.02200000000000002</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>17</v>
@@ -823,10 +823,10 @@
         <v>2255</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>8659494.359999999</v>
+        <v>8652050.039999999</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>1247634.31</v>
+        <v>1245567.76</v>
       </c>
       <c r="J7" s="6">
         <f>IF(H7=0,"",I7/H7)</f>
@@ -836,7 +836,7 @@
         <v>2285352</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>23</v>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="P7" s="6" t="n">
-        <v>0</v>
+        <v>0.03300000000000003</v>
       </c>
       <c r="Q7" s="4" t="n">
         <v>17</v>
@@ -965,7 +965,7 @@
         <v>39</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>992580.71</v>
+        <v>989602.99</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>244713.67</v>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0</v>
+        <v>0.04200000000000004</v>
       </c>
       <c r="Q9" s="4" t="n">
         <v>17</v>
@@ -1036,10 +1036,10 @@
         <v>1538</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>17529277.02</v>
+        <v>17527788.15</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>4024225.37</v>
+        <v>4023812.06</v>
       </c>
       <c r="J10" s="6">
         <f>IF(H10=0,"",I10/H10)</f>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>17</v>
@@ -1249,10 +1249,10 @@
         <v>232</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>5788034.84</v>
+        <v>5700020.48</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1381203.09</v>
+        <v>1356770.31</v>
       </c>
       <c r="J13" s="6">
         <f>IF(H13=0,"",I13/H13)</f>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0</v>
+        <v>0.05900000000000005</v>
       </c>
       <c r="Q13" s="4" t="n">
         <v>17</v>
@@ -1320,10 +1320,10 @@
         <v>2660</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>31866716.63</v>
+        <v>31836939.35</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>7428998.04</v>
+        <v>7420731.87</v>
       </c>
       <c r="J14" s="6">
         <f>IF(H14=0,"",I14/H14)</f>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="P14" s="6" t="n">
-        <v>0</v>
+        <v>0.01200000000000001</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>17</v>
@@ -1391,10 +1391,10 @@
         <v>2268</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>30585796.02</v>
+        <v>30527838.53</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>7274410.75</v>
+        <v>7258321.76</v>
       </c>
       <c r="J15" s="6">
         <f>IF(H15=0,"",I15/H15)</f>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="P15" s="6" t="n">
-        <v>0.04500000000000004</v>
+        <v>0.05000000000000004</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>17</v>
@@ -1462,10 +1462,10 @@
         <v>98</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>3059085.94</v>
+        <v>3025050.32</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>745653.99</v>
+        <v>736205.7</v>
       </c>
       <c r="J16" s="6">
         <f>IF(H16=0,"",I16/H16)</f>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="P16" s="6" t="n">
-        <v>0</v>
+        <v>0.05800000000000005</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>17</v>
@@ -1533,10 +1533,10 @@
         <v>2266</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>11079390.78</v>
+        <v>9544151.92</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>1657249.58</v>
+        <v>1568259.8</v>
       </c>
       <c r="J17" s="6">
         <f>IF(H17=0,"",I17/H17)</f>
@@ -1546,13 +1546,13 @@
         <v>2492632.28</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>21</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>0.322</v>
+        <v>0.343</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="P17" s="6" t="n">
-        <v>0.01800000000000002</v>
+        <v>0.5509999999999999</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>17</v>
@@ -1604,10 +1604,10 @@
         <v>106</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>4759969.53</v>
+        <v>4674678.59</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1160418.11</v>
+        <v>1136741.34</v>
       </c>
       <c r="J18" s="6">
         <f>IF(H18=0,"",I18/H18)</f>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0.03700000000000003</v>
+        <v>0.111</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>17</v>
@@ -1746,10 +1746,10 @@
         <v>98</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>2786213.1</v>
+        <v>2771269.98</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>669904.49</v>
+        <v>665756.28</v>
       </c>
       <c r="J20" s="6">
         <f>IF(H20=0,"",I20/H20)</f>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="P20" s="6" t="n">
-        <v>0</v>
+        <v>0.08299999999999996</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>17</v>
@@ -1817,10 +1817,10 @@
         <v>1928</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>21150658.08</v>
+        <v>21144690.36</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>4776250.77</v>
+        <v>4774594.13</v>
       </c>
       <c r="J21" s="6">
         <f>IF(H21=0,"",I21/H21)</f>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="P21" s="6" t="n">
-        <v>0.229</v>
+        <v>0.231</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>17</v>
@@ -1888,10 +1888,10 @@
         <v>1769</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>11633057.47</v>
+        <v>11630858.38</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>2575776.17</v>
+        <v>2575165.71</v>
       </c>
       <c r="J22" s="6">
         <f>IF(H22=0,"",I22/H22)</f>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0</v>
+        <v>0.004000000000000004</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>17</v>
@@ -1959,10 +1959,10 @@
         <v>76</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>3147880.1</v>
+        <v>3140600.5</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>834882.85</v>
+        <v>832862.03</v>
       </c>
       <c r="J23" s="6">
         <f>IF(H23=0,"",I23/H23)</f>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="P23" s="6" t="n">
-        <v>0</v>
+        <v>0.02000000000000002</v>
       </c>
       <c r="Q23" s="4" t="n">
         <v>17</v>
@@ -2172,10 +2172,10 @@
         <v>2914</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>19497183.25</v>
+        <v>19147742.96</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>3864978.19</v>
+        <v>3767973.57</v>
       </c>
       <c r="J26" s="6">
         <f>IF(H26=0,"",I26/H26)</f>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.02300000000000002</v>
       </c>
       <c r="Q26" s="4" t="n">
         <v>17</v>
@@ -2456,10 +2456,10 @@
         <v>3385</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>36794481</v>
+        <v>37430393.58</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>8425204.869999999</v>
+        <v>8601734.199999999</v>
       </c>
       <c r="J30" s="6">
         <f>IF(H30=0,"",I30/H30)</f>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="P30" s="6" t="n">
-        <v>0</v>
+        <v>0.661</v>
       </c>
       <c r="Q30" s="4" t="n">
         <v>17</v>
@@ -2527,10 +2527,10 @@
         <v>1273</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>6528520.26</v>
+        <v>6531734.23</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>1159592.08</v>
+        <v>1160484.27</v>
       </c>
       <c r="J31" s="6">
         <f>IF(H31=0,"",I31/H31)</f>
@@ -2554,7 +2554,7 @@
         </is>
       </c>
       <c r="P31" s="6" t="n">
-        <v>0.01000000000000001</v>
+        <v>0.153</v>
       </c>
       <c r="Q31" s="4" t="n">
         <v>17</v>
@@ -2598,10 +2598,10 @@
         <v>41</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>682859.98</v>
+        <v>675430.89</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>168539.36</v>
+        <v>166477.05</v>
       </c>
       <c r="J32" s="6">
         <f>IF(H32=0,"",I32/H32)</f>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0</v>
+        <v>0.03400000000000003</v>
       </c>
       <c r="Q32" s="4" t="n">
         <v>17</v>
@@ -2669,10 +2669,10 @@
         <v>2762</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>13002327.96</v>
+        <v>12758906.54</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>2086644.49</v>
+        <v>2019070.71</v>
       </c>
       <c r="J33" s="6">
         <f>IF(H33=0,"",I33/H33)</f>
@@ -2682,13 +2682,13 @@
         <v>2551248</v>
       </c>
       <c r="L33" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M33" s="7" t="n">
         <v>25</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>0.326</v>
+        <v>0.325</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -2696,7 +2696,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n">
-        <v>0.03400000000000003</v>
+        <v>0.141</v>
       </c>
       <c r="Q33" s="4" t="n">
         <v>17</v>
@@ -2811,10 +2811,10 @@
         <v>6061</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>28128304</v>
+        <v>27033676.25</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>4594067.71</v>
+        <v>4290199.05</v>
       </c>
       <c r="J35" s="6">
         <f>IF(H35=0,"",I35/H35)</f>
@@ -2824,13 +2824,13 @@
         <v>5725224</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M35" s="7" t="n">
         <v>55</v>
       </c>
       <c r="N35" s="8" t="n">
-        <v>0.326</v>
+        <v>0.325</v>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="P35" s="6" t="n">
-        <v>0</v>
+        <v>0.265</v>
       </c>
       <c r="Q35" s="4" t="n">
         <v>17</v>
@@ -2882,10 +2882,10 @@
         <v>16671</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>81967734.19</v>
+        <v>65839101.18</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>15308095.98</v>
+        <v>10830787.46</v>
       </c>
       <c r="J36" s="6">
         <f>IF(H36=0,"",I36/H36)</f>
@@ -2895,13 +2895,13 @@
         <v>13714242.99</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="M36" s="7" t="n">
         <v>151</v>
       </c>
       <c r="N36" s="8" t="n">
-        <v>0.333</v>
+        <v>0.326</v>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0</v>
+        <v>0.6990000000000001</v>
       </c>
       <c r="Q36" s="4" t="n">
         <v>17</v>
@@ -2953,10 +2953,10 @@
         <v>1491</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>12936989.02</v>
+        <v>12775674.03</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>2636748.2</v>
+        <v>2591967.15</v>
       </c>
       <c r="J37" s="6">
         <f>IF(H37=0,"",I37/H37)</f>
@@ -2972,7 +2972,7 @@
         <v>15</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>0.338</v>
+        <v>0.337</v>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.858</v>
+        <v>0.92</v>
       </c>
       <c r="Q37" s="4" t="n">
         <v>17</v>
@@ -3024,10 +3024,10 @@
         <v>292</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>11678474.51</v>
+        <v>11593125.27</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>2962843.96</v>
+        <v>2939151.01</v>
       </c>
       <c r="J38" s="6">
         <f>IF(H38=0,"",I38/H38)</f>
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="P38" s="6" t="n">
-        <v>0.02600000000000002</v>
+        <v>0.06999999999999995</v>
       </c>
       <c r="Q38" s="4" t="n">
         <v>17</v>
@@ -3095,10 +3095,10 @@
         <v>912</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>5634188.81</v>
+        <v>5417814.21</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>956016.26</v>
+        <v>895950.67</v>
       </c>
       <c r="J39" s="6">
         <f>IF(H39=0,"",I39/H39)</f>
@@ -3108,13 +3108,13 @@
         <v>987808.49</v>
       </c>
       <c r="L39" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M39" s="7" t="n">
         <v>8</v>
       </c>
       <c r="N39" s="8" t="n">
-        <v>0.33</v>
+        <v>0.329</v>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.261</v>
+        <v>0.478</v>
       </c>
       <c r="Q39" s="4" t="n">
         <v>17</v>
@@ -3166,10 +3166,10 @@
         <v>125</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>4424642.29</v>
+        <v>4345263.33</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>1042418.88</v>
+        <v>1020383.28</v>
       </c>
       <c r="J40" s="6">
         <f>IF(H40=0,"",I40/H40)</f>
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="P40" s="6" t="n">
-        <v>0</v>
+        <v>0.04900000000000004</v>
       </c>
       <c r="Q40" s="4" t="n">
         <v>17</v>
@@ -3237,10 +3237,10 @@
         <v>106</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1634821.48</v>
+        <v>1330261.85</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>360052.33</v>
+        <v>299945.21</v>
       </c>
       <c r="J41" s="6">
         <f>IF(H41=0,"",I41/H41)</f>
@@ -3256,7 +3256,7 @@
         <v>2</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>0.344</v>
+        <v>0.467</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         </is>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.06100000000000005</v>
+        <v>0.198</v>
       </c>
       <c r="Q41" s="4" t="n">
         <v>16</v>
@@ -3308,10 +3308,10 @@
         <v>1419</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>7662037.48</v>
+        <v>7600305.07</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>1215512.89</v>
+        <v>1198375.97</v>
       </c>
       <c r="J42" s="6">
         <f>IF(H42=0,"",I42/H42)</f>
@@ -3327,7 +3327,7 @@
         <v>13</v>
       </c>
       <c r="N42" s="8" t="n">
-        <v>0.326</v>
+        <v>0.325</v>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="P42" s="6" t="n">
-        <v>0.284</v>
+        <v>0.3139999999999999</v>
       </c>
       <c r="Q42" s="4" t="n">
         <v>17</v>
@@ -3379,7 +3379,7 @@
         <v>3419</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>12272260.2</v>
+        <v>12239938.18</v>
       </c>
       <c r="I43" s="5" t="n">
         <v>1949285.51</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="P43" s="6" t="n">
-        <v>0.03700000000000003</v>
+        <v>0.04900000000000004</v>
       </c>
       <c r="Q43" s="4" t="n">
         <v>17</v>
@@ -3450,10 +3450,10 @@
         <v>502</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>13615381.15</v>
+        <v>13262726.72</v>
       </c>
       <c r="I44" s="5" t="n">
-        <v>3415633.12</v>
+        <v>3317736.25</v>
       </c>
       <c r="J44" s="6">
         <f>IF(H44=0,"",I44/H44)</f>
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="P44" s="6" t="n">
-        <v>0.03800000000000003</v>
+        <v>0.122</v>
       </c>
       <c r="Q44" s="4" t="n">
         <v>17</v>
@@ -3521,10 +3521,10 @@
         <v>235</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>4493834.23</v>
+        <v>3935375.68</v>
       </c>
       <c r="I45" s="5" t="n">
-        <v>1096096.07</v>
+        <v>941067.97</v>
       </c>
       <c r="J45" s="6">
         <f>IF(H45=0,"",I45/H45)</f>
@@ -3540,7 +3540,7 @@
         <v>3</v>
       </c>
       <c r="N45" s="8" t="n">
-        <v>0.346</v>
+        <v>0.345</v>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         </is>
       </c>
       <c r="P45" s="6" t="n">
-        <v>0</v>
+        <v>0.872</v>
       </c>
       <c r="Q45" s="4" t="n">
         <v>17</v>
@@ -3592,10 +3592,10 @@
         <v>3940</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>21814060.42</v>
+        <v>19084116.27</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>3635322.5</v>
+        <v>3553706.38</v>
       </c>
       <c r="J46" s="6">
         <f>IF(H46=0,"",I46/H46)</f>
@@ -3605,13 +3605,13 @@
         <v>4337146.55</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M46" s="7" t="n">
         <v>36</v>
       </c>
       <c r="N46" s="8" t="n">
-        <v>0.327</v>
+        <v>0.38</v>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="P46" s="6" t="n">
-        <v>0.03500000000000003</v>
+        <v>0.329</v>
       </c>
       <c r="Q46" s="4" t="n">
         <v>17</v>
@@ -3663,7 +3663,7 @@
         <v>3261</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>10954055.03</v>
+        <v>10952685.28</v>
       </c>
       <c r="I47" s="5" t="n">
         <v>1640998.99</v>
@@ -3690,7 +3690,7 @@
         </is>
       </c>
       <c r="P47" s="6" t="n">
-        <v>0</v>
+        <v>0.006000000000000005</v>
       </c>
       <c r="Q47" s="4" t="n">
         <v>17</v>
@@ -3734,10 +3734,10 @@
         <v>65</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>2779745.33</v>
+        <v>2762186.59</v>
       </c>
       <c r="I48" s="5" t="n">
-        <v>770833.72</v>
+        <v>765959.41</v>
       </c>
       <c r="J48" s="6">
         <f>IF(H48=0,"",I48/H48)</f>
@@ -3761,7 +3761,7 @@
         </is>
       </c>
       <c r="P48" s="6" t="n">
-        <v>0.007000000000000006</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="Q48" s="4" t="n">
         <v>17</v>
@@ -3805,10 +3805,10 @@
         <v>208</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>4789794.63</v>
+        <v>4722081.52</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1116397.5</v>
+        <v>1097600.34</v>
       </c>
       <c r="J49" s="6">
         <f>IF(H49=0,"",I49/H49)</f>
@@ -3824,7 +3824,7 @@
         <v>3</v>
       </c>
       <c r="N49" s="8" t="n">
-        <v>0.346</v>
+        <v>0.345</v>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="P49" s="6" t="n">
-        <v>0.07399999999999995</v>
+        <v>0.116</v>
       </c>
       <c r="Q49" s="4" t="n">
         <v>17</v>
@@ -3876,10 +3876,10 @@
         <v>134</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>1923460.09</v>
+        <v>1885106.05</v>
       </c>
       <c r="I50" s="5" t="n">
-        <v>427672.13</v>
+        <v>417025.05</v>
       </c>
       <c r="J50" s="6">
         <f>IF(H50=0,"",I50/H50)</f>
@@ -3903,7 +3903,7 @@
         </is>
       </c>
       <c r="P50" s="6" t="n">
-        <v>0</v>
+        <v>0.03500000000000003</v>
       </c>
       <c r="Q50" s="4" t="n">
         <v>17</v>
@@ -3947,10 +3947,10 @@
         <v>1089</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>22704990.14</v>
+        <v>21820648.8</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>5770071.55</v>
+        <v>5524578.4</v>
       </c>
       <c r="J51" s="6">
         <f>IF(H51=0,"",I51/H51)</f>
@@ -3974,7 +3974,7 @@
         </is>
       </c>
       <c r="P51" s="6" t="n">
-        <v>0</v>
+        <v>0.06100000000000005</v>
       </c>
       <c r="Q51" s="4" t="n">
         <v>17</v>
@@ -4018,10 +4018,10 @@
         <v>835</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>4699559.06</v>
+        <v>3847343.12</v>
       </c>
       <c r="I52" s="5" t="n">
-        <v>885213.67</v>
+        <v>648638.52</v>
       </c>
       <c r="J52" s="6">
         <f>IF(H52=0,"",I52/H52)</f>
@@ -4031,13 +4031,13 @@
         <v>686712.52</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="M52" s="7" t="n">
         <v>8</v>
       </c>
       <c r="N52" s="8" t="n">
-        <v>0.335</v>
+        <v>0.33</v>
       </c>
       <c r="O52" s="4" t="inlineStr">
         <is>
@@ -4045,7 +4045,7 @@
         </is>
       </c>
       <c r="P52" s="6" t="n">
-        <v>0</v>
+        <v>0.601</v>
       </c>
       <c r="Q52" s="4" t="n">
         <v>17</v>
@@ -4089,10 +4089,10 @@
         <v>181</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>6228675.04</v>
+        <v>6180254.35</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>1529674.84</v>
+        <v>1516233.25</v>
       </c>
       <c r="J53" s="6">
         <f>IF(H53=0,"",I53/H53)</f>
@@ -4116,7 +4116,7 @@
         </is>
       </c>
       <c r="P53" s="6" t="n">
-        <v>0</v>
+        <v>0.02000000000000002</v>
       </c>
       <c r="Q53" s="4" t="n">
         <v>17</v>
@@ -4160,10 +4160,10 @@
         <v>1363</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>6323454.09</v>
+        <v>5269388.71</v>
       </c>
       <c r="I54" s="5" t="n">
-        <v>1312676.97</v>
+        <v>1020068.42</v>
       </c>
       <c r="J54" s="6">
         <f>IF(H54=0,"",I54/H54)</f>
@@ -4173,13 +4173,13 @@
         <v>758181.9</v>
       </c>
       <c r="L54" s="7" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M54" s="7" t="n">
         <v>13</v>
       </c>
       <c r="N54" s="8" t="n">
-        <v>0.338</v>
+        <v>0.335</v>
       </c>
       <c r="O54" s="4" t="inlineStr">
         <is>
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="P54" s="6" t="n">
-        <v>0</v>
+        <v>0.3110000000000001</v>
       </c>
       <c r="Q54" s="4" t="n">
         <v>17</v>
@@ -4369,16 +4369,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2905267.73</v>
+        <v>2907843.4</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0</v>
+        <v>0.09799999999999998</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.9571</v>
+        <v>0.9584</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -4387,7 +4387,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.0429</v>
+        <v>0.0416</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>0</v>
@@ -4411,16 +4411,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1168338.17</v>
+        <v>1159918.54</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0</v>
+        <v>0.02200000000000002</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.866</v>
+        <v>0.8723</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -4429,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.134</v>
+        <v>0.1277</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>0</v>
@@ -4453,16 +4453,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8659494.359999999</v>
+        <v>8652050.039999999</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0</v>
+        <v>0.03300000000000003</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.9251</v>
+        <v>0.9258999999999999</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -4471,7 +4471,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.07489999999999999</v>
+        <v>0.0741</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>0</v>
@@ -4537,16 +4537,16 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>992580.71</v>
+        <v>989602.99</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>0.04200000000000004</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.953</v>
+        <v>0.9559</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -4555,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.047</v>
+        <v>0.0441</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0</v>
@@ -4579,16 +4579,16 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>17529277.02</v>
+        <v>17527788.15</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>0.009979999999999999</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>0.001000000000000001</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.9349</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -4597,7 +4597,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.06510000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
@@ -4705,16 +4705,16 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5788034.84</v>
+        <v>5700020.48</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>0</v>
+        <v>0.05900000000000005</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.8025</v>
+        <v>0.8148</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -4723,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.1975</v>
+        <v>0.1852</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>0</v>
@@ -4747,16 +4747,16 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>31866716.63</v>
+        <v>31836939.35</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0</v>
+        <v>0.01200000000000001</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0.9265</v>
+        <v>0.9274</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>0</v>
@@ -4765,7 +4765,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.0735</v>
+        <v>0.0726</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>0</v>
@@ -4789,16 +4789,16 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>30585796.02</v>
+        <v>30527838.53</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.04500000000000004</v>
+        <v>0.05000000000000004</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.9595</v>
+        <v>0.9613</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>0</v>
@@ -4807,7 +4807,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.0405</v>
+        <v>0.0387</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0</v>
@@ -4831,16 +4831,16 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>3059085.94</v>
+        <v>3025050.32</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0</v>
+        <v>0.05800000000000005</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0.8885</v>
+        <v>0.8985</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>0</v>
@@ -4849,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.1115</v>
+        <v>0.1015</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>0</v>
@@ -4873,16 +4873,16 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>11079390.78</v>
+        <v>9544151.92</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.01800000000000002</v>
+        <v>0.5509999999999999</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9386</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -4891,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.0529</v>
+        <v>0.0614</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0</v>
@@ -4915,16 +4915,16 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>4759969.53</v>
+        <v>4674678.59</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.00899</v>
+        <v>0.008970000000000001</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.03700000000000003</v>
+        <v>0.111</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>0.8263</v>
+        <v>0.8414</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>0</v>
@@ -4933,7 +4933,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.1737</v>
+        <v>0.1586</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
@@ -4999,16 +4999,16 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>2786213.1</v>
+        <v>2771269.98</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0</v>
+        <v>0.08299999999999996</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9401</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>0</v>
@@ -5017,7 +5017,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.065</v>
+        <v>0.0599</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
@@ -5041,16 +5041,16 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>21150658.08</v>
+        <v>21144690.36</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>0.229</v>
+        <v>0.231</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.95</v>
+        <v>0.9503</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
@@ -5059,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.05</v>
+        <v>0.0497</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
@@ -5083,16 +5083,16 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11633057.47</v>
+        <v>11630858.38</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>0</v>
+        <v>0.004000000000000004</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.9423</v>
+        <v>0.9425</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>0</v>
@@ -5101,7 +5101,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.0577</v>
+        <v>0.0575</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
@@ -5125,16 +5125,16 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3147880.1</v>
+        <v>3140600.5</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>0</v>
+        <v>0.02000000000000002</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.9545</v>
+        <v>0.9567</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
@@ -5143,7 +5143,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.0455</v>
+        <v>0.0433</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
@@ -5251,16 +5251,16 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>19497183.25</v>
+        <v>19147742.96</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.02300000000000002</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>0.9486</v>
+        <v>0.966</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>0</v>
@@ -5269,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.0514</v>
+        <v>0.034</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0</v>
@@ -5419,16 +5419,16 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>36794481</v>
+        <v>37430393.58</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0</v>
+        <v>0.661</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0.9520999999999999</v>
+        <v>0.9469</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>0</v>
@@ -5437,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.0479</v>
+        <v>0.0531</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>0</v>
@@ -5461,16 +5461,16 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>6528520.26</v>
+        <v>6531734.23</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>0.01000000000000001</v>
+        <v>0.153</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>0.8793</v>
+        <v>0.8789</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>0</v>
@@ -5479,7 +5479,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.1207</v>
+        <v>0.1211</v>
       </c>
       <c r="I31" s="6" t="n">
         <v>0</v>
@@ -5503,16 +5503,16 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>682859.98</v>
+        <v>675430.89</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>0</v>
+        <v>0.03400000000000003</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.882</v>
+        <v>0.8917</v>
       </c>
       <c r="F32" s="6" t="n">
         <v>0</v>
@@ -5521,7 +5521,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.118</v>
+        <v>0.1083</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0</v>
@@ -5545,16 +5545,16 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>13002327.96</v>
+        <v>12758906.54</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>0.03400000000000003</v>
+        <v>0.141</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.9273</v>
+        <v>0.926</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -5563,7 +5563,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.0727</v>
+        <v>0.074</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
@@ -5629,16 +5629,16 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>28128304</v>
+        <v>27033676.25</v>
       </c>
       <c r="C35" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>0</v>
+        <v>0.265</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>0.9362</v>
+        <v>0.9337</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -5647,7 +5647,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0.0638</v>
+        <v>0.0663</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>0</v>
@@ -5671,16 +5671,16 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>81967734.19</v>
+        <v>65839101.18</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>0</v>
+        <v>0.6990000000000001</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0.9374</v>
+        <v>0.9221</v>
       </c>
       <c r="F36" s="6" t="n">
         <v>0</v>
@@ -5689,7 +5689,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.0626</v>
+        <v>0.0779</v>
       </c>
       <c r="I36" s="6" t="n">
         <v>0</v>
@@ -5713,16 +5713,16 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>12936989.02</v>
+        <v>12775674.03</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>0.858</v>
+        <v>0.92</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9508</v>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
@@ -5731,7 +5731,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0.061</v>
+        <v>0.0492</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0</v>
@@ -5755,16 +5755,16 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>11678474.51</v>
+        <v>11593125.27</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>0.02600000000000002</v>
+        <v>0.06999999999999995</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.9016999999999999</v>
+        <v>0.9083</v>
       </c>
       <c r="F38" s="6" t="n">
         <v>0</v>
@@ -5773,7 +5773,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.0983</v>
+        <v>0.0917</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>
@@ -5797,16 +5797,16 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5634188.81</v>
+        <v>5417814.21</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>0.261</v>
+        <v>0.478</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.9292</v>
       </c>
       <c r="F39" s="6" t="n">
         <v>0</v>
@@ -5815,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.068</v>
+        <v>0.0708</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
@@ -5839,16 +5839,16 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>4424642.29</v>
+        <v>4345263.33</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>0</v>
+        <v>0.04900000000000004</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0.8092</v>
+        <v>0.824</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
@@ -5857,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0.1908</v>
+        <v>0.176</v>
       </c>
       <c r="I40" s="6" t="n">
         <v>0</v>
@@ -5881,16 +5881,16 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1634821.48</v>
+        <v>1330261.85</v>
       </c>
       <c r="C41" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>0.06100000000000005</v>
+        <v>0.198</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>0.9332</v>
+        <v>0.9179</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
@@ -5899,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.0668</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>
@@ -5923,16 +5923,16 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7662037.48</v>
+        <v>7600305.07</v>
       </c>
       <c r="C42" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>0.284</v>
+        <v>0.3139999999999999</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0.9554</v>
+        <v>0.9631999999999999</v>
       </c>
       <c r="F42" s="6" t="n">
         <v>0</v>
@@ -5941,7 +5941,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.0446</v>
+        <v>0.0368</v>
       </c>
       <c r="I42" s="6" t="n">
         <v>0</v>
@@ -5965,16 +5965,16 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>12272260.2</v>
+        <v>12239938.18</v>
       </c>
       <c r="C43" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>0.03700000000000003</v>
+        <v>0.04900000000000004</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>0.9638</v>
+        <v>0.9637</v>
       </c>
       <c r="F43" s="6" t="n">
         <v>0</v>
@@ -5983,7 +5983,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>0.0362</v>
+        <v>0.0363</v>
       </c>
       <c r="I43" s="6" t="n">
         <v>0</v>
@@ -6007,16 +6007,16 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>13615381.15</v>
+        <v>13262726.72</v>
       </c>
       <c r="C44" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>0.03800000000000003</v>
+        <v>0.122</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>0.6418</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="F44" s="6" t="n">
         <v>0</v>
@@ -6025,7 +6025,7 @@
         <v>0</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0.3582</v>
+        <v>0.3412</v>
       </c>
       <c r="I44" s="6" t="n">
         <v>0</v>
@@ -6049,16 +6049,16 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>4493834.23</v>
+        <v>3935375.68</v>
       </c>
       <c r="C45" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>0</v>
+        <v>0.872</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>0.9566</v>
+        <v>0.9557</v>
       </c>
       <c r="F45" s="6" t="n">
         <v>0</v>
@@ -6067,7 +6067,7 @@
         <v>0</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>0.0434</v>
+        <v>0.0443</v>
       </c>
       <c r="I45" s="6" t="n">
         <v>0</v>
@@ -6091,16 +6091,16 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>21814060.42</v>
+        <v>19084116.27</v>
       </c>
       <c r="C46" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>0.03500000000000003</v>
+        <v>0.329</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>0.9508</v>
+        <v>0.9438</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>0</v>
@@ -6109,7 +6109,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.0492</v>
+        <v>0.0562</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>0</v>
@@ -6133,16 +6133,16 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>10954055.03</v>
+        <v>10952685.28</v>
       </c>
       <c r="C47" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>0</v>
+        <v>0.006000000000000005</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>0.9688</v>
+        <v>0.9689</v>
       </c>
       <c r="F47" s="6" t="n">
         <v>0</v>
@@ -6151,7 +6151,7 @@
         <v>0</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>0.0312</v>
+        <v>0.0311</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>0</v>
@@ -6175,16 +6175,16 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>2779745.33</v>
+        <v>2762186.59</v>
       </c>
       <c r="C48" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>0.007000000000000006</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>0.9162</v>
+        <v>0.9221</v>
       </c>
       <c r="F48" s="6" t="n">
         <v>0</v>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.0838</v>
+        <v>0.0779</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
@@ -6217,16 +6217,16 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>4789794.63</v>
+        <v>4722081.52</v>
       </c>
       <c r="C49" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>0.07399999999999995</v>
+        <v>0.116</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>0.8207</v>
+        <v>0.8324</v>
       </c>
       <c r="F49" s="6" t="n">
         <v>0</v>
@@ -6235,7 +6235,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.1793</v>
+        <v>0.1676</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>0</v>
@@ -6259,16 +6259,16 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>1923460.09</v>
+        <v>1885106.05</v>
       </c>
       <c r="C50" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>0</v>
+        <v>0.03500000000000003</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>0.9253</v>
+        <v>0.9441000000000001</v>
       </c>
       <c r="F50" s="6" t="n">
         <v>0</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.0747</v>
+        <v>0.0559</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>0</v>
@@ -6301,16 +6301,16 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>22704990.14</v>
+        <v>21820648.8</v>
       </c>
       <c r="C51" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>0</v>
+        <v>0.06100000000000005</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>0.9141</v>
+        <v>0.9512</v>
       </c>
       <c r="F51" s="6" t="n">
         <v>0</v>
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.0859</v>
+        <v>0.0488</v>
       </c>
       <c r="I51" s="6" t="n">
         <v>0</v>
@@ -6343,16 +6343,16 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>4699559.06</v>
+        <v>3847343.12</v>
       </c>
       <c r="C52" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>0</v>
+        <v>0.601</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>0.9411</v>
+        <v>0.9281</v>
       </c>
       <c r="F52" s="6" t="n">
         <v>0</v>
@@ -6361,7 +6361,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.0589</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="I52" s="6" t="n">
         <v>0</v>
@@ -6385,16 +6385,16 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>6228675.04</v>
+        <v>6180254.35</v>
       </c>
       <c r="C53" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>0</v>
+        <v>0.02000000000000002</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>0.7667</v>
+        <v>0.7727000000000001</v>
       </c>
       <c r="F53" s="6" t="n">
         <v>0</v>
@@ -6403,7 +6403,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.2333</v>
+        <v>0.2273</v>
       </c>
       <c r="I53" s="6" t="n">
         <v>0</v>
@@ -6427,16 +6427,16 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>6323454.09</v>
+        <v>5269388.71</v>
       </c>
       <c r="C54" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>0</v>
+        <v>0.3110000000000001</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>0.9101</v>
+        <v>0.8921</v>
       </c>
       <c r="F54" s="6" t="n">
         <v>0</v>
@@ -6445,7 +6445,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.08989999999999999</v>
+        <v>0.1079</v>
       </c>
       <c r="I54" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on the Spanish DIA 100 rate
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The register held through the run
- 28 approved, 21 revoked, 10 undecided.

The set baseline moves from EUR 584,087,950 to 566,908,926 (-17.2M,
-2.9%) across three companies, matching what the rate was priced at
before the change: Santander -12.8M (-42%), Fresenius -4.2M, Carrefour
-0.1M. Best-case saving falls 4.8M to 112.4M, and Santander's
steady-state payback goes from 11 months to 20. Sourced prices now carry
25.3% of priced value, up from 22.5%. The other 47 companies change only
in run ids and timestamps; 49 stay COMPLETE for their declared scope and
Capgemini PARTIAL, as before.

The price review is rebuilt on the new card. ES-DIA-100-researched now
stands against the EUR 250 rate, and approving it would take a further
EUR 2.4M off.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -1391,10 +1391,10 @@
         <v>2268</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>30527838.53</v>
+        <v>17697685.39</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>7258321.76</v>
+        <v>3696671.24</v>
       </c>
       <c r="J15" s="6">
         <f>IF(H15=0,"",I15/H15)</f>
@@ -1404,13 +1404,13 @@
         <v>2576016</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>28</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>0.343</v>
+        <v>0.338</v>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="P15" s="6" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.552</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>17</v>
@@ -1675,10 +1675,10 @@
         <v>8982</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>39900513.72</v>
+        <v>39782444.83</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>6417602.43</v>
+        <v>6384826.51</v>
       </c>
       <c r="J19" s="6">
         <f>IF(H19=0,"",I19/H19)</f>
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0</v>
+        <v>0.003000000000000003</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>17</v>
@@ -2456,10 +2456,10 @@
         <v>3385</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>37430393.58</v>
+        <v>33199591.55</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>8601734.199999999</v>
+        <v>7427263.56</v>
       </c>
       <c r="J30" s="6">
         <f>IF(H30=0,"",I30/H30)</f>
@@ -2469,13 +2469,13 @@
         <v>3492648</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M30" s="7" t="n">
         <v>36</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>0.342</v>
+        <v>0.341</v>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="P30" s="6" t="n">
-        <v>0.661</v>
+        <v>0.846</v>
       </c>
       <c r="Q30" s="4" t="n">
         <v>17</v>
@@ -4789,16 +4789,16 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>30527838.53</v>
+        <v>17697685.39</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.552</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.9613</v>
+        <v>0.9333</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>0</v>
@@ -4807,7 +4807,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.0387</v>
+        <v>0.0667</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0</v>
@@ -4957,16 +4957,16 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>39900513.72</v>
+        <v>39782444.83</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0</v>
+        <v>0.003000000000000003</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9369</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
@@ -4975,7 +4975,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.063</v>
+        <v>0.0631</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
@@ -5419,16 +5419,16 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>37430393.58</v>
+        <v>33199591.55</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.661</v>
+        <v>0.846</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0.9469</v>
+        <v>0.9401</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>0</v>
@@ -5437,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.0531</v>
+        <v>0.0599</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on the UK DIA 500 rate
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The register held through the run
- 28 approved, 25 revoked, 6 undecided - and research challenged five
decisions with other figures, which the card did not take.

The set baseline moves from EUR 566,908,926 to 566,093,106 (-0.82M)
across six companies, exactly what was priced before the change:
Deutsche Post DHL -662k, Royal Mail -95k, UPS -40k, Tesco -14k, Boots
-3k, McDonald's -1k. Best-case saving falls 0.22M to 112.2M. Sourced
prices now carry 26.6% of priced value, up from 25.3%. No circuit in the
set prices at GB DIA 300, so its repricing moves nothing. The other 44
companies change only in run ids and timestamps; 49 stay COMPLETE for
their declared scope and Capgemini PARTIAL, as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -1533,7 +1533,7 @@
         <v>2266</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>9544151.92</v>
+        <v>9540989.82</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>1568259.8</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="P17" s="6" t="n">
-        <v>0.5509999999999999</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>17</v>
@@ -2172,10 +2172,10 @@
         <v>2914</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>19147742.96</v>
+        <v>18485284.48</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>3767973.57</v>
+        <v>3584075.09</v>
       </c>
       <c r="J26" s="6">
         <f>IF(H26=0,"",I26/H26)</f>
@@ -2185,13 +2185,13 @@
         <v>2779632</v>
       </c>
       <c r="L26" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M26" s="7" t="n">
         <v>27</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>0.336</v>
+        <v>0.335</v>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.02300000000000002</v>
+        <v>0.3139999999999999</v>
       </c>
       <c r="Q26" s="4" t="n">
         <v>17</v>
@@ -2882,10 +2882,10 @@
         <v>16671</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>65839101.18</v>
+        <v>65837836.35</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>10830787.46</v>
+        <v>10830436.34</v>
       </c>
       <c r="J36" s="6">
         <f>IF(H36=0,"",I36/H36)</f>
@@ -3308,10 +3308,10 @@
         <v>1419</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>7600305.07</v>
+        <v>7504809.87</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>1198375.97</v>
+        <v>1171866.51</v>
       </c>
       <c r="J42" s="6">
         <f>IF(H42=0,"",I42/H42)</f>
@@ -3321,7 +3321,7 @@
         <v>1549785.3</v>
       </c>
       <c r="L42" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M42" s="7" t="n">
         <v>13</v>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="P42" s="6" t="n">
-        <v>0.3139999999999999</v>
+        <v>0.484</v>
       </c>
       <c r="Q42" s="4" t="n">
         <v>17</v>
@@ -3592,7 +3592,7 @@
         <v>3940</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>19084116.27</v>
+        <v>19070203.07</v>
       </c>
       <c r="I46" s="5" t="n">
         <v>3553706.38</v>
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="P46" s="6" t="n">
-        <v>0.329</v>
+        <v>0.342</v>
       </c>
       <c r="Q46" s="4" t="n">
         <v>17</v>
@@ -3947,10 +3947,10 @@
         <v>1089</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>21820648.8</v>
+        <v>21781122.63</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>5524578.4</v>
+        <v>5513605.93</v>
       </c>
       <c r="J51" s="6">
         <f>IF(H51=0,"",I51/H51)</f>
@@ -3974,7 +3974,7 @@
         </is>
       </c>
       <c r="P51" s="6" t="n">
-        <v>0.06100000000000005</v>
+        <v>0.07099999999999995</v>
       </c>
       <c r="Q51" s="4" t="n">
         <v>17</v>
@@ -4873,16 +4873,16 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>9544151.92</v>
+        <v>9540989.82</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.5509999999999999</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>0.9386</v>
+        <v>0.9389</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -4891,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.0614</v>
+        <v>0.0611</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0</v>
@@ -5251,16 +5251,16 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>19147742.96</v>
+        <v>18485284.48</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0.02300000000000002</v>
+        <v>0.3139999999999999</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>0.966</v>
+        <v>0.9647</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>0</v>
@@ -5269,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.034</v>
+        <v>0.0353</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0</v>
@@ -5671,7 +5671,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>65839101.18</v>
+        <v>65837836.35</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>0.01</v>
@@ -5923,16 +5923,16 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7600305.07</v>
+        <v>7504809.87</v>
       </c>
       <c r="C42" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>0.3139999999999999</v>
+        <v>0.484</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0.9631999999999999</v>
+        <v>0.964</v>
       </c>
       <c r="F42" s="6" t="n">
         <v>0</v>
@@ -5941,7 +5941,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.0368</v>
+        <v>0.036</v>
       </c>
       <c r="I42" s="6" t="n">
         <v>0</v>
@@ -6091,16 +6091,16 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>19084116.27</v>
+        <v>19070203.07</v>
       </c>
       <c r="C46" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>0.329</v>
+        <v>0.342</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>0.9438</v>
+        <v>0.9444</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>0</v>
@@ -6109,7 +6109,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.0562</v>
+        <v>0.0556</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>0</v>
@@ -6301,16 +6301,16 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>21820648.8</v>
+        <v>21781122.63</v>
       </c>
       <c r="C51" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>0.06100000000000005</v>
+        <v>0.07099999999999995</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>0.9512</v>
+        <v>0.9510999999999999</v>
       </c>
       <c r="F51" s="6" t="n">
         <v>0</v>
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.0488</v>
+        <v>0.0489</v>
       </c>
       <c r="I51" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on Singapore's 5G prices
No provider calls: the same research, re-promoted and re-estimated on the
new card. Only DBS moves. Its 1,100 ATMs' 5G line falls from SGD 1.05M to
SGD 0.39M a year, its baseline by SGD 658,944 (3.9%) to SGD 16.43M, and
its best-case saving from SGD 3.78M to 3.60M.

The set falls EUR 448,442 to EUR 576,794,766, best-case saving EUR
124,488 to EUR 115,176,662, and sourced prices carry 27.1% of priced
value. The other 49 companies change only in run ids, timestamps and the
order of their footprint rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-set-summary.xlsx
+++ b/docs/sample-set-summary.xlsx
@@ -1888,10 +1888,10 @@
         <v>1769</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>11630858.38</v>
+        <v>11182416.1</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>2575165.71</v>
+        <v>2450678.12</v>
       </c>
       <c r="J22" s="6">
         <f>IF(H22=0,"",I22/H22)</f>
@@ -1901,13 +1901,13 @@
         <v>1242183.16</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>19</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>0.341</v>
+        <v>0.34</v>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.03900000000000003</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>17</v>
@@ -5083,16 +5083,16 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11630858.38</v>
+        <v>11182416.1</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>0.004000000000000004</v>
+        <v>0.03900000000000003</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.9425</v>
+        <v>0.9402</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>0</v>
@@ -5101,7 +5101,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.0575</v>
+        <v>0.0598</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>

</xml_diff>